<commit_message>
debug + data elec
</commit_message>
<xml_diff>
--- a/inventories/lci-Tr2050.xlsx
+++ b/inventories/lci-Tr2050.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joanna.schlesinger\0.Joanna\2. HySPI\ADEME_scenarios_premise\inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7AB6699-6060-4CC3-AB5A-19744D2ED2F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2C6A939-99C3-4F15-BC92-E69198D11B9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -341,10 +341,10 @@
     <t>market for electricity, high voltage</t>
   </si>
   <si>
+    <t>electricity production, from stationary battery, Tr2050</t>
+  </si>
+  <si>
     <t>Tr2050</t>
-  </si>
-  <si>
-    <t>electricity production, from stationary battery, Tr2050</t>
   </si>
 </sst>
 </file>
@@ -840,7 +840,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
@@ -2167,7 +2167,7 @@
         <v>1</v>
       </c>
       <c r="B78" s="12" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C78" s="13"/>
       <c r="D78" s="9"/>

</xml_diff>

<commit_message>
error on flow location
</commit_message>
<xml_diff>
--- a/inventories/lci-Tr2050.xlsx
+++ b/inventories/lci-Tr2050.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27531"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joanna.schlesinger\0.Joanna\2. HySPI\ADEME_scenarios_premise\inventories\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jschlesinger\0.Joanna\2. HySPI\ADEME_scenarios_premise\inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{020733DF-B953-436F-BEDB-05172F433018}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6DA717C-3527-4B78-8471-A05AD2896F12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="lci" sheetId="1" r:id="rId1"/>
@@ -2986,7 +2986,7 @@
         <v>108</v>
       </c>
       <c r="D109" s="43" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E109" s="43" t="s">
         <v>13</v>
@@ -4062,7 +4062,7 @@
         <v>108</v>
       </c>
       <c r="D157" s="43" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E157" s="43" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
delete market H2 fossil fuel refinery because of unexplained error + creation of empty inventory
</commit_message>
<xml_diff>
--- a/inventories/lci-Tr2050.xlsx
+++ b/inventories/lci-Tr2050.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jschlesinger\0.Joanna\2. HySPI\ADEME_scenarios_premise\inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1521C391-BCF6-4923-B754-ECBD64DA2349}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A46D53F0-D429-4579-B7F6-F2E75EEE23EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="lci" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="884" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="909" uniqueCount="198">
   <si>
     <t>Database</t>
   </si>
@@ -625,6 +625,15 @@
   </si>
   <si>
     <t>electricity production, hydro, pumped storage, Tr2050</t>
+  </si>
+  <si>
+    <t>nothing</t>
+  </si>
+  <si>
+    <t>empty activity, for market that does not exist any more in 2050, Tr2050</t>
+  </si>
+  <si>
+    <t>used for market for hydrogen, for fossil fuel refinery in 2050 as this market does not exist anymore in 2050</t>
   </si>
 </sst>
 </file>
@@ -1119,7 +1128,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T166"/>
+  <dimension ref="A1:T185"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="55.36328125" customWidth="1"/>
@@ -4578,6 +4587,144 @@
       </c>
       <c r="I166" s="43"/>
     </row>
+    <row r="168" spans="1:9" ht="15.5">
+      <c r="A168" s="34" t="s">
+        <v>1</v>
+      </c>
+      <c r="B168" s="34" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="169" spans="1:9">
+      <c r="A169" t="s">
+        <v>2</v>
+      </c>
+      <c r="B169" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="170" spans="1:9">
+      <c r="A170" t="s">
+        <v>11</v>
+      </c>
+      <c r="B170" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="171" spans="1:9">
+      <c r="A171" t="s">
+        <v>3</v>
+      </c>
+      <c r="B171">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="172" spans="1:9">
+      <c r="A172" t="s">
+        <v>76</v>
+      </c>
+      <c r="B172"/>
+    </row>
+    <row r="173" spans="1:9">
+      <c r="A173" t="s">
+        <v>4</v>
+      </c>
+      <c r="B173" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="174" spans="1:9">
+      <c r="A174" t="s">
+        <v>5</v>
+      </c>
+      <c r="B174" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="175" spans="1:9">
+      <c r="A175" t="s">
+        <v>6</v>
+      </c>
+      <c r="B175" s="43" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="176" spans="1:9" ht="15.5">
+      <c r="A176" s="34" t="s">
+        <v>7</v>
+      </c>
+      <c r="B176"/>
+    </row>
+    <row r="177" spans="1:8" ht="15.5">
+      <c r="A177" s="34" t="s">
+        <v>8</v>
+      </c>
+      <c r="B177" s="34" t="s">
+        <v>9</v>
+      </c>
+      <c r="C177" s="34" t="s">
+        <v>2</v>
+      </c>
+      <c r="D177" s="34" t="s">
+        <v>6</v>
+      </c>
+      <c r="E177" s="34" t="s">
+        <v>10</v>
+      </c>
+      <c r="F177" s="34" t="s">
+        <v>5</v>
+      </c>
+      <c r="G177" s="34" t="s">
+        <v>4</v>
+      </c>
+      <c r="H177" s="34" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="178" spans="1:8">
+      <c r="A178" t="str">
+        <f>B168</f>
+        <v>empty activity, for market that does not exist any more in 2050, Tr2050</v>
+      </c>
+      <c r="B178">
+        <v>1</v>
+      </c>
+      <c r="C178" t="s">
+        <v>29</v>
+      </c>
+      <c r="D178" t="str">
+        <f>B175</f>
+        <v>kilogram</v>
+      </c>
+      <c r="F178" t="s">
+        <v>18</v>
+      </c>
+      <c r="G178" t="str">
+        <f>B173</f>
+        <v>nothing</v>
+      </c>
+    </row>
+    <row r="179" spans="1:8">
+      <c r="B179"/>
+    </row>
+    <row r="180" spans="1:8">
+      <c r="B180" s="41"/>
+    </row>
+    <row r="181" spans="1:8">
+      <c r="B181" s="41"/>
+    </row>
+    <row r="182" spans="1:8">
+      <c r="B182" s="41"/>
+    </row>
+    <row r="183" spans="1:8">
+      <c r="B183"/>
+    </row>
+    <row r="184" spans="1:8">
+      <c r="B184"/>
+    </row>
+    <row r="185" spans="1:8">
+      <c r="B185"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Corrected gas burned in the network to be included within the 1.5% losses rate Modified gas burning for biomethane to consider the French activity of heat production from biomethane
</commit_message>
<xml_diff>
--- a/inventories/lci-Tr2050.xlsx
+++ b/inventories/lci-Tr2050.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://engie-my.sharepoint.com/personal/db6421_engie_com/Documents/Documents/GitHub/ADEME_scenarios_premise_gas/inventories/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1718" documentId="13_ncr:1_{6A9A1C53-53B4-4DAF-B82F-70FF83AECA95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0FDF5E9E-0A4E-4357-85CA-802D21303263}"/>
+  <xr:revisionPtr revIDLastSave="1759" documentId="13_ncr:1_{6A9A1C53-53B4-4DAF-B82F-70FF83AECA95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D0D3474-BBD2-4870-A7ED-E2183A0A0CA7}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="lci" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3936" uniqueCount="482">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3934" uniqueCount="480">
   <si>
     <t>Database</t>
   </si>
@@ -815,9 +815,6 @@
     <t>biomethane AD transport</t>
   </si>
   <si>
-    <t>market for heat, central or small-scale, biomethane</t>
-  </si>
-  <si>
     <t>heat, central or small-scale, biomethane</t>
   </si>
   <si>
@@ -950,21 +947,12 @@
     <t>Import of biomethane (anaerobic digestion and gasification of wood)</t>
   </si>
   <si>
-    <t>5.93e-03 MJ heat/MJ natural gas high pressure (Faist Emmenegger et al., 2017). Biomethane LHV = 34.72 MJ considering a constant upgrading mix</t>
-  </si>
-  <si>
     <t>Scaled to reference product based on ecoinvent Faist Emmenegger M., Del Duce A., Moreno Ruiz E., Brunner F., (2017). Update of the European natural gas supply chains. Ecoinvent, Zürich, Switzerland</t>
   </si>
   <si>
     <t>market for biogas</t>
   </si>
   <si>
-    <t>5.93e-03 MJ heat/MJ natural gas high pressure (Faist Emmenegger et al., 2017).LHV = 35</t>
-  </si>
-  <si>
-    <t>1.5% of losses (ADEME Transition 2050)</t>
-  </si>
-  <si>
     <t>1.5% ADEME Transition 2050. Calculated from the estimated composition of biomethane from AD in the French mix after upgrading</t>
   </si>
   <si>
@@ -1482,6 +1470,12 @@
   </si>
   <si>
     <t>platinum group metal, extraction and refinery operations</t>
+  </si>
+  <si>
+    <t>1.5% of losses including the burned natural gas (ADEME Transition 2050)</t>
+  </si>
+  <si>
+    <t>heat production, biomethane, at boiler condensing modulating &lt;100kW</t>
   </si>
 </sst>
 </file>
@@ -1638,7 +1632,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -1720,6 +1714,7 @@
     <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1739,10 +1734,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2009,17 +2000,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AH923"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="73.109375" customWidth="1"/>
-    <col min="2" max="2" width="18.5546875" style="13" customWidth="1"/>
-    <col min="3" max="3" width="17.109375" customWidth="1"/>
-    <col min="4" max="4" width="24.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.44140625" customWidth="1"/>
-    <col min="6" max="6" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="33.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.5546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="109.6640625" customWidth="1"/>
+    <col min="1" max="1" width="73.140625" customWidth="1"/>
+    <col min="2" max="2" width="18.5703125" style="13" customWidth="1"/>
+    <col min="3" max="3" width="17.140625" customWidth="1"/>
+    <col min="4" max="4" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.42578125" customWidth="1"/>
+    <col min="6" max="6" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="109.7109375" customWidth="1"/>
     <col min="10" max="10" width="31" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2071,7 +2062,7 @@
       <c r="I4" s="6"/>
       <c r="K4" s="5"/>
     </row>
-    <row r="5" spans="1:14" ht="15.6">
+    <row r="5" spans="1:14" ht="15.75">
       <c r="A5" s="18" t="s">
         <v>1</v>
       </c>
@@ -2153,7 +2144,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="15.6">
+    <row r="13" spans="1:14" ht="15.75">
       <c r="A13" s="18" t="s">
         <v>7</v>
       </c>
@@ -2162,7 +2153,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="14" spans="1:14" ht="15.6">
+    <row r="14" spans="1:14" ht="15.75">
       <c r="A14" s="18" t="s">
         <v>8</v>
       </c>
@@ -2875,7 +2866,7 @@
       <c r="AG47" s="47"/>
       <c r="AH47" s="47"/>
     </row>
-    <row r="48" spans="1:34" s="15" customFormat="1" ht="15.6">
+    <row r="48" spans="1:34" s="15" customFormat="1" ht="15.75">
       <c r="A48" s="2" t="s">
         <v>1</v>
       </c>
@@ -2895,7 +2886,7 @@
       <c r="O48" s="16"/>
       <c r="P48" s="16"/>
     </row>
-    <row r="49" spans="1:20" s="15" customFormat="1" ht="15.6">
+    <row r="49" spans="1:20" s="15" customFormat="1" ht="15.75">
       <c r="A49" s="2" t="s">
         <v>3</v>
       </c>
@@ -2915,7 +2906,7 @@
       <c r="O49" s="16"/>
       <c r="P49" s="16"/>
     </row>
-    <row r="50" spans="1:20" s="15" customFormat="1" ht="15.6">
+    <row r="50" spans="1:20" s="15" customFormat="1" ht="15.75">
       <c r="A50" s="2" t="s">
         <v>11</v>
       </c>
@@ -2935,7 +2926,7 @@
       <c r="O50" s="16"/>
       <c r="P50" s="16"/>
     </row>
-    <row r="51" spans="1:20" s="15" customFormat="1" ht="15.6">
+    <row r="51" spans="1:20" s="15" customFormat="1" ht="15.75">
       <c r="A51" s="2" t="s">
         <v>4</v>
       </c>
@@ -2955,7 +2946,7 @@
       <c r="O51" s="16"/>
       <c r="P51" s="16"/>
     </row>
-    <row r="52" spans="1:20" s="15" customFormat="1" ht="15.6">
+    <row r="52" spans="1:20" s="15" customFormat="1" ht="15.75">
       <c r="A52" s="2" t="s">
         <v>2</v>
       </c>
@@ -2975,7 +2966,7 @@
       <c r="O52" s="16"/>
       <c r="P52" s="16"/>
     </row>
-    <row r="53" spans="1:20" s="15" customFormat="1" ht="15.6">
+    <row r="53" spans="1:20" s="15" customFormat="1" ht="15.75">
       <c r="A53" s="2" t="s">
         <v>6</v>
       </c>
@@ -2997,7 +2988,7 @@
       <c r="O53" s="16"/>
       <c r="P53" s="16"/>
     </row>
-    <row r="54" spans="1:20" s="15" customFormat="1" ht="15.6">
+    <row r="54" spans="1:20" s="15" customFormat="1" ht="15.75">
       <c r="A54" s="2" t="s">
         <v>7</v>
       </c>
@@ -3017,7 +3008,7 @@
       <c r="O54" s="16"/>
       <c r="P54" s="16"/>
     </row>
-    <row r="55" spans="1:20" s="15" customFormat="1" ht="15.6">
+    <row r="55" spans="1:20" s="15" customFormat="1" ht="15.75">
       <c r="A55" s="2" t="s">
         <v>8</v>
       </c>
@@ -3055,7 +3046,7 @@
       <c r="S55" s="17"/>
       <c r="T55" s="18"/>
     </row>
-    <row r="56" spans="1:20" s="15" customFormat="1" ht="15.6">
+    <row r="56" spans="1:20" s="15" customFormat="1" ht="15.75">
       <c r="A56" t="s">
         <v>54</v>
       </c>
@@ -3087,7 +3078,7 @@
       <c r="P56" s="16"/>
       <c r="T56"/>
     </row>
-    <row r="57" spans="1:20" s="15" customFormat="1" ht="15.6">
+    <row r="57" spans="1:20" s="15" customFormat="1" ht="15.75">
       <c r="A57" t="s">
         <v>52</v>
       </c>
@@ -3121,7 +3112,7 @@
       <c r="Q57"/>
       <c r="R57"/>
     </row>
-    <row r="58" spans="1:20" s="15" customFormat="1" ht="15.6">
+    <row r="58" spans="1:20" s="15" customFormat="1" ht="15.75">
       <c r="A58" t="s">
         <v>53</v>
       </c>
@@ -3155,7 +3146,7 @@
       <c r="Q58"/>
       <c r="R58"/>
     </row>
-    <row r="59" spans="1:20" s="15" customFormat="1" ht="15.6">
+    <row r="59" spans="1:20" s="15" customFormat="1" ht="15.75">
       <c r="A59" t="s">
         <v>43</v>
       </c>
@@ -3189,7 +3180,7 @@
       <c r="Q59"/>
       <c r="R59"/>
     </row>
-    <row r="60" spans="1:20" s="15" customFormat="1" ht="15.6">
+    <row r="60" spans="1:20" s="15" customFormat="1" ht="15.75">
       <c r="A60" t="s">
         <v>46</v>
       </c>
@@ -3223,7 +3214,7 @@
       <c r="Q60"/>
       <c r="R60"/>
     </row>
-    <row r="61" spans="1:20" s="15" customFormat="1" ht="15.6">
+    <row r="61" spans="1:20" s="15" customFormat="1" ht="15.75">
       <c r="A61" t="s">
         <v>27</v>
       </c>
@@ -3256,7 +3247,7 @@
       <c r="Q61"/>
       <c r="R61"/>
     </row>
-    <row r="62" spans="1:20" s="15" customFormat="1" ht="15.6">
+    <row r="62" spans="1:20" s="15" customFormat="1" ht="15.75">
       <c r="A62" t="s">
         <v>21</v>
       </c>
@@ -3289,7 +3280,7 @@
       <c r="Q62"/>
       <c r="R62"/>
     </row>
-    <row r="63" spans="1:20" s="15" customFormat="1" ht="15.6">
+    <row r="63" spans="1:20" s="15" customFormat="1" ht="15.75">
       <c r="A63" t="s">
         <v>24</v>
       </c>
@@ -3318,7 +3309,7 @@
       <c r="Q63" s="20"/>
       <c r="R63"/>
     </row>
-    <row r="64" spans="1:20" s="15" customFormat="1" ht="15.6">
+    <row r="64" spans="1:20" s="15" customFormat="1" ht="15.75">
       <c r="A64" t="s">
         <v>51</v>
       </c>
@@ -3387,7 +3378,7 @@
       <c r="AG65" s="47"/>
       <c r="AH65" s="47"/>
     </row>
-    <row r="66" spans="1:34" ht="15.6">
+    <row r="66" spans="1:34" ht="15.75">
       <c r="A66" s="18" t="s">
         <v>1</v>
       </c>
@@ -3449,13 +3440,13 @@
         <v>13</v>
       </c>
     </row>
-    <row r="74" spans="1:34" ht="15.6">
+    <row r="74" spans="1:34" ht="15.75">
       <c r="A74" s="18" t="s">
         <v>7</v>
       </c>
       <c r="B74"/>
     </row>
-    <row r="75" spans="1:34" ht="15.6">
+    <row r="75" spans="1:34" ht="15.75">
       <c r="A75" s="18" t="s">
         <v>8</v>
       </c>
@@ -3585,7 +3576,7 @@
         <v>11</v>
       </c>
       <c r="B79" s="26" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="C79" s="25"/>
       <c r="D79" s="26"/>
@@ -4691,7 +4682,7 @@
         <v>11</v>
       </c>
       <c r="B103" s="26" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="C103" s="25"/>
       <c r="D103" s="26"/>
@@ -5747,7 +5738,7 @@
         <v>11</v>
       </c>
       <c r="B126" s="26" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="C126" s="25"/>
       <c r="D126" s="26"/>
@@ -6803,7 +6794,7 @@
         <v>11</v>
       </c>
       <c r="B149" s="26" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="C149" s="25"/>
       <c r="D149" s="26"/>
@@ -7887,7 +7878,7 @@
         <v>11</v>
       </c>
       <c r="B173" s="26" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="C173" s="25"/>
       <c r="D173" s="26"/>
@@ -8756,7 +8747,7 @@
         <v>11</v>
       </c>
       <c r="B197" s="26" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="C197" s="25"/>
       <c r="D197" s="26"/>
@@ -9133,10 +9124,10 @@
     </row>
     <row r="206" spans="1:34">
       <c r="A206" s="26" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B206" s="26" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C206" s="32">
         <v>5.2260830394610069</v>
@@ -9791,7 +9782,7 @@
         <v>11</v>
       </c>
       <c r="B221" s="26" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="C221" s="25"/>
       <c r="D221" s="26"/>
@@ -10605,7 +10596,7 @@
         <v>11</v>
       </c>
       <c r="B245" s="26" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="C245" s="25"/>
       <c r="D245" s="26"/>
@@ -11384,7 +11375,7 @@
         <v>1</v>
       </c>
       <c r="B268" s="24" t="s">
-        <v>424</v>
+        <v>420</v>
       </c>
       <c r="C268" s="22"/>
       <c r="D268" s="22"/>
@@ -11444,7 +11435,7 @@
         <v>4</v>
       </c>
       <c r="B271" s="22" t="s">
-        <v>423</v>
+        <v>419</v>
       </c>
       <c r="C271" s="22"/>
       <c r="D271" s="22"/>
@@ -11464,7 +11455,7 @@
         <v>57</v>
       </c>
       <c r="B272" s="31" t="s">
-        <v>429</v>
+        <v>425</v>
       </c>
       <c r="C272" s="22"/>
       <c r="D272" s="22"/>
@@ -11548,10 +11539,10 @@
     </row>
     <row r="276" spans="1:14">
       <c r="A276" s="22" t="s">
-        <v>424</v>
+        <v>420</v>
       </c>
       <c r="B276" s="22" t="s">
-        <v>423</v>
+        <v>419</v>
       </c>
       <c r="C276" s="22">
         <v>1</v>
@@ -11574,10 +11565,10 @@
     </row>
     <row r="277" spans="1:14">
       <c r="A277" s="22" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="B277" s="22" t="s">
-        <v>338</v>
+        <v>334</v>
       </c>
       <c r="C277" s="22">
         <v>8.9499999999999996E-3</v>
@@ -11596,7 +11587,7 @@
         <v>12</v>
       </c>
       <c r="I277" s="22" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
       <c r="K277" s="22"/>
       <c r="L277" s="22"/>
@@ -11605,7 +11596,7 @@
     </row>
     <row r="278" spans="1:14">
       <c r="A278" s="22" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B278" s="22" t="s">
         <v>99</v>
@@ -11627,7 +11618,7 @@
         <v>12</v>
       </c>
       <c r="I278" s="22" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="K278" s="22"/>
       <c r="L278" s="22"/>
@@ -11658,7 +11649,7 @@
         <v>12</v>
       </c>
       <c r="I279" s="22" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="K279" s="22"/>
       <c r="L279" s="22"/>
@@ -11667,10 +11658,10 @@
     </row>
     <row r="280" spans="1:14">
       <c r="A280" s="22" t="s">
-        <v>341</v>
+        <v>337</v>
       </c>
       <c r="B280" s="22" t="s">
-        <v>343</v>
+        <v>339</v>
       </c>
       <c r="C280" s="22">
         <v>1.79E-6</v>
@@ -11689,7 +11680,7 @@
         <v>12</v>
       </c>
       <c r="I280" s="22" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="K280" s="22"/>
       <c r="L280" s="22"/>
@@ -11698,10 +11689,10 @@
     </row>
     <row r="281" spans="1:14">
       <c r="A281" s="22" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="B281" s="22" t="s">
-        <v>346</v>
+        <v>342</v>
       </c>
       <c r="C281" s="22">
         <v>9.859999999999999E-4</v>
@@ -11720,7 +11711,7 @@
         <v>12</v>
       </c>
       <c r="I281" s="22" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
       <c r="K281" s="22"/>
       <c r="L281" s="22"/>
@@ -11729,10 +11720,10 @@
     </row>
     <row r="282" spans="1:14">
       <c r="A282" s="22" t="s">
-        <v>347</v>
+        <v>343</v>
       </c>
       <c r="B282" s="22" t="s">
-        <v>349</v>
+        <v>345</v>
       </c>
       <c r="C282" s="22">
         <v>5.3699999999999998E-3</v>
@@ -11751,7 +11742,7 @@
         <v>12</v>
       </c>
       <c r="I282" s="22" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
       <c r="K282" s="22"/>
       <c r="L282" s="22"/>
@@ -11760,10 +11751,10 @@
     </row>
     <row r="283" spans="1:14">
       <c r="A283" s="22" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="B283" s="22" t="s">
-        <v>352</v>
+        <v>348</v>
       </c>
       <c r="C283" s="22">
         <v>5.3699999999999998E-3</v>
@@ -11782,7 +11773,7 @@
         <v>12</v>
       </c>
       <c r="I283" s="22" t="s">
-        <v>351</v>
+        <v>347</v>
       </c>
       <c r="K283" s="22"/>
       <c r="L283" s="22"/>
@@ -11791,10 +11782,10 @@
     </row>
     <row r="284" spans="1:14">
       <c r="A284" s="22" t="s">
-        <v>353</v>
+        <v>349</v>
       </c>
       <c r="B284" s="22" t="s">
-        <v>354</v>
+        <v>350</v>
       </c>
       <c r="C284" s="22">
         <v>2.3300000000000001E-2</v>
@@ -11813,7 +11804,7 @@
         <v>12</v>
       </c>
       <c r="I284" s="22" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="K284" s="22"/>
       <c r="L284" s="22"/>
@@ -11822,10 +11813,10 @@
     </row>
     <row r="285" spans="1:14">
       <c r="A285" s="22" t="s">
-        <v>355</v>
+        <v>351</v>
       </c>
       <c r="B285" s="22" t="s">
-        <v>357</v>
+        <v>353</v>
       </c>
       <c r="C285" s="22">
         <v>0.55700000000000005</v>
@@ -11844,7 +11835,7 @@
         <v>12</v>
       </c>
       <c r="I285" s="22" t="s">
-        <v>356</v>
+        <v>352</v>
       </c>
       <c r="K285" s="22"/>
       <c r="L285" s="22"/>
@@ -11875,7 +11866,7 @@
         <v>12</v>
       </c>
       <c r="I286" s="22" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="K286" s="22"/>
       <c r="L286" s="22"/>
@@ -11906,7 +11897,7 @@
         <v>12</v>
       </c>
       <c r="I287" s="22" t="s">
-        <v>359</v>
+        <v>355</v>
       </c>
       <c r="K287" s="22"/>
       <c r="L287" s="22"/>
@@ -11915,10 +11906,10 @@
     </row>
     <row r="288" spans="1:14">
       <c r="A288" s="22" t="s">
-        <v>360</v>
+        <v>356</v>
       </c>
       <c r="B288" s="22" t="s">
-        <v>361</v>
+        <v>357</v>
       </c>
       <c r="C288" s="22">
         <v>3.9199999999999999E-3</v>
@@ -11937,7 +11928,7 @@
         <v>12</v>
       </c>
       <c r="I288" s="22" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="K288" s="22"/>
       <c r="L288" s="22"/>
@@ -11966,7 +11957,7 @@
         <v>15</v>
       </c>
       <c r="I289" s="22" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="K289" s="22"/>
       <c r="L289" s="22"/>
@@ -11995,7 +11986,7 @@
         <v>15</v>
       </c>
       <c r="I290" s="22" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
       <c r="K290" s="22"/>
       <c r="L290" s="22"/>
@@ -12004,7 +11995,7 @@
     </row>
     <row r="291" spans="1:14">
       <c r="A291" s="22" t="s">
-        <v>362</v>
+        <v>358</v>
       </c>
       <c r="C291" s="22">
         <v>15.4</v>
@@ -12017,13 +12008,13 @@
       </c>
       <c r="F291" s="22"/>
       <c r="G291" s="22" t="s">
-        <v>363</v>
+        <v>359</v>
       </c>
       <c r="H291" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I291" s="22" t="s">
-        <v>364</v>
+        <v>360</v>
       </c>
       <c r="J291" s="22"/>
       <c r="K291" s="22"/>
@@ -12052,7 +12043,7 @@
         <v>15</v>
       </c>
       <c r="I292" s="22" t="s">
-        <v>422</v>
+        <v>418</v>
       </c>
       <c r="J292" s="22"/>
       <c r="K292" s="22"/>
@@ -12062,7 +12053,7 @@
     </row>
     <row r="293" spans="1:14">
       <c r="A293" s="22" t="s">
-        <v>365</v>
+        <v>361</v>
       </c>
       <c r="C293" s="22">
         <v>1.4</v>
@@ -12081,7 +12072,7 @@
         <v>15</v>
       </c>
       <c r="I293" s="22" t="s">
-        <v>366</v>
+        <v>362</v>
       </c>
       <c r="J293" s="22"/>
       <c r="K293" s="22"/>
@@ -12091,7 +12082,7 @@
     </row>
     <row r="294" spans="1:14">
       <c r="A294" s="22" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C294" s="22">
         <v>1.4</v>
@@ -12110,7 +12101,7 @@
         <v>15</v>
       </c>
       <c r="I294" s="22" t="s">
-        <v>368</v>
+        <v>364</v>
       </c>
       <c r="J294" s="22"/>
       <c r="K294" s="22"/>
@@ -12120,7 +12111,7 @@
     </row>
     <row r="295" spans="1:14">
       <c r="A295" s="22" t="s">
-        <v>369</v>
+        <v>365</v>
       </c>
       <c r="C295" s="22">
         <v>1.4</v>
@@ -12139,7 +12130,7 @@
         <v>15</v>
       </c>
       <c r="I295" s="22" t="s">
-        <v>368</v>
+        <v>364</v>
       </c>
       <c r="J295" s="22"/>
       <c r="K295" s="22"/>
@@ -12168,7 +12159,7 @@
         <v>15</v>
       </c>
       <c r="I296" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J296" s="22"/>
       <c r="K296" s="22"/>
@@ -12197,7 +12188,7 @@
         <v>15</v>
       </c>
       <c r="I297" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J297" s="22"/>
       <c r="K297" s="22"/>
@@ -12226,7 +12217,7 @@
         <v>15</v>
       </c>
       <c r="I298" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J298" s="22"/>
       <c r="K298" s="22"/>
@@ -12236,7 +12227,7 @@
     </row>
     <row r="299" spans="1:14">
       <c r="A299" s="22" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
       <c r="C299" s="22">
         <v>0.48</v>
@@ -12255,7 +12246,7 @@
         <v>15</v>
       </c>
       <c r="I299" s="22" t="s">
-        <v>372</v>
+        <v>368</v>
       </c>
       <c r="J299" s="22"/>
       <c r="K299" s="22"/>
@@ -12265,7 +12256,7 @@
     </row>
     <row r="300" spans="1:14">
       <c r="A300" s="22" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
       <c r="C300" s="22">
         <v>0.48</v>
@@ -12284,7 +12275,7 @@
         <v>15</v>
       </c>
       <c r="I300" s="22" t="s">
-        <v>372</v>
+        <v>368</v>
       </c>
       <c r="J300" s="22"/>
       <c r="K300" s="22"/>
@@ -12294,7 +12285,7 @@
     </row>
     <row r="301" spans="1:14">
       <c r="A301" s="22" t="s">
-        <v>374</v>
+        <v>370</v>
       </c>
       <c r="C301" s="22">
         <v>0.96</v>
@@ -12313,7 +12304,7 @@
         <v>15</v>
       </c>
       <c r="I301" s="22" t="s">
-        <v>375</v>
+        <v>371</v>
       </c>
       <c r="J301" s="22"/>
       <c r="K301" s="22"/>
@@ -12323,7 +12314,7 @@
     </row>
     <row r="302" spans="1:14">
       <c r="A302" s="22" t="s">
-        <v>376</v>
+        <v>372</v>
       </c>
       <c r="C302" s="22">
         <v>1.0100000000000001E-6</v>
@@ -12336,13 +12327,13 @@
       </c>
       <c r="F302" s="22"/>
       <c r="G302" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H302" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I302" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J302" s="22"/>
       <c r="K302" s="22"/>
@@ -12352,7 +12343,7 @@
     </row>
     <row r="303" spans="1:14">
       <c r="A303" s="22" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="C303" s="22">
         <v>6.1399999999999997E-7</v>
@@ -12365,13 +12356,13 @@
       </c>
       <c r="F303" s="22"/>
       <c r="G303" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H303" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I303" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J303" s="22"/>
       <c r="K303" s="22"/>
@@ -12381,7 +12372,7 @@
     </row>
     <row r="304" spans="1:14">
       <c r="A304" s="22" t="s">
-        <v>379</v>
+        <v>375</v>
       </c>
       <c r="C304" s="22">
         <v>4.8099999999999997E-9</v>
@@ -12394,13 +12385,13 @@
       </c>
       <c r="F304" s="22"/>
       <c r="G304" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H304" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I304" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J304" s="22"/>
       <c r="K304" s="22"/>
@@ -12410,7 +12401,7 @@
     </row>
     <row r="305" spans="1:14">
       <c r="A305" s="22" t="s">
-        <v>380</v>
+        <v>376</v>
       </c>
       <c r="C305" s="22">
         <v>6.5000000000000002E-7</v>
@@ -12423,13 +12414,13 @@
       </c>
       <c r="F305" s="22"/>
       <c r="G305" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H305" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I305" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J305" s="22"/>
       <c r="K305" s="22"/>
@@ -12439,7 +12430,7 @@
     </row>
     <row r="306" spans="1:14">
       <c r="A306" s="22" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="C306" s="22">
         <v>-1.5E-6</v>
@@ -12452,13 +12443,13 @@
       </c>
       <c r="F306" s="22"/>
       <c r="G306" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H306" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I306" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J306" s="22"/>
       <c r="K306" s="22"/>
@@ -12468,7 +12459,7 @@
     </row>
     <row r="307" spans="1:14">
       <c r="A307" s="22" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="C307" s="22">
         <v>1.1999999999999999E-7</v>
@@ -12481,13 +12472,13 @@
       </c>
       <c r="F307" s="22"/>
       <c r="G307" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H307" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I307" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J307" s="22"/>
       <c r="K307" s="22"/>
@@ -12497,7 +12488,7 @@
     </row>
     <row r="308" spans="1:14">
       <c r="A308" s="22" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
       <c r="C308" s="22">
         <v>2.48E-6</v>
@@ -12510,13 +12501,13 @@
       </c>
       <c r="F308" s="22"/>
       <c r="G308" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H308" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I308" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J308" s="22"/>
       <c r="K308" s="22"/>
@@ -12526,7 +12517,7 @@
     </row>
     <row r="309" spans="1:14">
       <c r="A309" s="22" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="C309" s="22">
         <v>1.08E-7</v>
@@ -12539,13 +12530,13 @@
       </c>
       <c r="F309" s="22"/>
       <c r="G309" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H309" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I309" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J309" s="22"/>
       <c r="K309" s="22"/>
@@ -12555,7 +12546,7 @@
     </row>
     <row r="310" spans="1:14">
       <c r="A310" s="22" t="s">
-        <v>385</v>
+        <v>381</v>
       </c>
       <c r="C310" s="22">
         <v>1.0100000000000001E-6</v>
@@ -12568,13 +12559,13 @@
       </c>
       <c r="F310" s="22"/>
       <c r="G310" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H310" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I310" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J310" s="22"/>
       <c r="K310" s="22"/>
@@ -12584,7 +12575,7 @@
     </row>
     <row r="311" spans="1:14">
       <c r="A311" s="22" t="s">
-        <v>386</v>
+        <v>382</v>
       </c>
       <c r="C311" s="22">
         <v>2.4100000000000001E-8</v>
@@ -12597,13 +12588,13 @@
       </c>
       <c r="F311" s="22"/>
       <c r="G311" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H311" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I311" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J311" s="22"/>
       <c r="K311" s="22"/>
@@ -12613,7 +12604,7 @@
     </row>
     <row r="312" spans="1:14">
       <c r="A312" s="22" t="s">
-        <v>387</v>
+        <v>383</v>
       </c>
       <c r="C312" s="22">
         <v>-3.2899999999999999E-7</v>
@@ -12626,13 +12617,13 @@
       </c>
       <c r="F312" s="22"/>
       <c r="G312" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H312" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I312" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J312" s="22"/>
       <c r="K312" s="22"/>
@@ -12642,7 +12633,7 @@
     </row>
     <row r="313" spans="1:14">
       <c r="A313" s="22" t="s">
-        <v>388</v>
+        <v>384</v>
       </c>
       <c r="C313" s="22">
         <v>7.9400000000000004E-7</v>
@@ -12655,13 +12646,13 @@
       </c>
       <c r="F313" s="22"/>
       <c r="G313" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H313" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I313" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J313" s="22"/>
       <c r="K313" s="22"/>
@@ -12671,7 +12662,7 @@
     </row>
     <row r="314" spans="1:14">
       <c r="A314" s="22" t="s">
-        <v>389</v>
+        <v>385</v>
       </c>
       <c r="C314" s="22">
         <v>4.1400000000000002E-6</v>
@@ -12684,13 +12675,13 @@
       </c>
       <c r="F314" s="22"/>
       <c r="G314" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H314" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I314" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J314" s="22"/>
       <c r="K314" s="22"/>
@@ -12700,7 +12691,7 @@
     </row>
     <row r="315" spans="1:14">
       <c r="A315" s="22" t="s">
-        <v>390</v>
+        <v>386</v>
       </c>
       <c r="C315" s="22">
         <v>5.0500000000000002E-8</v>
@@ -12713,13 +12704,13 @@
       </c>
       <c r="F315" s="22"/>
       <c r="G315" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H315" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I315" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J315" s="22"/>
       <c r="K315" s="22"/>
@@ -12729,7 +12720,7 @@
     </row>
     <row r="316" spans="1:14">
       <c r="A316" s="22" t="s">
-        <v>391</v>
+        <v>387</v>
       </c>
       <c r="C316" s="22">
         <v>-5.9000000000000003E-6</v>
@@ -12742,13 +12733,13 @@
       </c>
       <c r="F316" s="22"/>
       <c r="G316" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H316" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I316" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J316" s="22"/>
       <c r="K316" s="22"/>
@@ -12758,7 +12749,7 @@
     </row>
     <row r="317" spans="1:14">
       <c r="A317" s="22" t="s">
-        <v>392</v>
+        <v>388</v>
       </c>
       <c r="C317" s="22">
         <v>1.5600000000000001E-6</v>
@@ -12771,13 +12762,13 @@
       </c>
       <c r="F317" s="22"/>
       <c r="G317" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H317" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I317" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J317" s="22"/>
       <c r="K317" s="22"/>
@@ -12787,7 +12778,7 @@
     </row>
     <row r="318" spans="1:14">
       <c r="A318" s="22" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
       <c r="C318" s="22">
         <v>2.7E-6</v>
@@ -12800,13 +12791,13 @@
       </c>
       <c r="F318" s="22"/>
       <c r="G318" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H318" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I318" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J318" s="22"/>
       <c r="K318" s="22"/>
@@ -12816,7 +12807,7 @@
     </row>
     <row r="319" spans="1:14">
       <c r="A319" s="22" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
       <c r="C319" s="22">
         <v>4.4500000000000001E-8</v>
@@ -12829,13 +12820,13 @@
       </c>
       <c r="F319" s="22"/>
       <c r="G319" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H319" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I319" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J319" s="22"/>
       <c r="K319" s="22"/>
@@ -12845,7 +12836,7 @@
     </row>
     <row r="320" spans="1:14">
       <c r="A320" s="22" t="s">
-        <v>395</v>
+        <v>391</v>
       </c>
       <c r="C320" s="22">
         <v>3.6099999999999999E-8</v>
@@ -12858,13 +12849,13 @@
       </c>
       <c r="F320" s="22"/>
       <c r="G320" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H320" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I320" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J320" s="22"/>
       <c r="K320" s="22"/>
@@ -12874,7 +12865,7 @@
     </row>
     <row r="321" spans="1:14">
       <c r="A321" s="22" t="s">
-        <v>396</v>
+        <v>392</v>
       </c>
       <c r="C321" s="22">
         <v>2.17E-7</v>
@@ -12887,13 +12878,13 @@
       </c>
       <c r="F321" s="22"/>
       <c r="G321" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H321" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I321" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J321" s="22"/>
       <c r="K321" s="22"/>
@@ -12903,7 +12894,7 @@
     </row>
     <row r="322" spans="1:14">
       <c r="A322" s="22" t="s">
-        <v>397</v>
+        <v>393</v>
       </c>
       <c r="C322" s="22">
         <v>-1.88E-8</v>
@@ -12916,13 +12907,13 @@
       </c>
       <c r="F322" s="22"/>
       <c r="G322" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H322" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I322" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J322" s="22"/>
       <c r="K322" s="22"/>
@@ -12932,7 +12923,7 @@
     </row>
     <row r="323" spans="1:14">
       <c r="A323" s="22" t="s">
-        <v>398</v>
+        <v>394</v>
       </c>
       <c r="C323" s="22">
         <v>4.2899999999999999E-5</v>
@@ -12945,13 +12936,13 @@
       </c>
       <c r="F323" s="22"/>
       <c r="G323" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H323" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I323" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J323" s="22"/>
       <c r="K323" s="22"/>
@@ -12961,7 +12952,7 @@
     </row>
     <row r="324" spans="1:14">
       <c r="A324" s="22" t="s">
-        <v>399</v>
+        <v>395</v>
       </c>
       <c r="C324" s="22">
         <v>9.2499999999999999E-5</v>
@@ -12974,13 +12965,13 @@
       </c>
       <c r="F324" s="22"/>
       <c r="G324" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H324" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I324" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J324" s="22"/>
       <c r="K324" s="22"/>
@@ -12990,7 +12981,7 @@
     </row>
     <row r="325" spans="1:14">
       <c r="A325" s="22" t="s">
-        <v>400</v>
+        <v>396</v>
       </c>
       <c r="C325" s="22">
         <v>5.0300000000000001E-6</v>
@@ -13003,13 +12994,13 @@
       </c>
       <c r="F325" s="22"/>
       <c r="G325" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H325" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I325" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J325" s="22"/>
       <c r="K325" s="22"/>
@@ -13019,7 +13010,7 @@
     </row>
     <row r="326" spans="1:14">
       <c r="A326" s="22" t="s">
-        <v>401</v>
+        <v>397</v>
       </c>
       <c r="C326" s="22">
         <v>2.43E-6</v>
@@ -13032,13 +13023,13 @@
       </c>
       <c r="F326" s="22"/>
       <c r="G326" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H326" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I326" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J326" s="22"/>
       <c r="K326" s="22"/>
@@ -13048,7 +13039,7 @@
     </row>
     <row r="327" spans="1:14">
       <c r="A327" s="22" t="s">
-        <v>402</v>
+        <v>398</v>
       </c>
       <c r="C327" s="22">
         <v>1.73E-6</v>
@@ -13061,13 +13052,13 @@
       </c>
       <c r="F327" s="22"/>
       <c r="G327" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H327" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I327" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J327" s="22"/>
       <c r="K327" s="22"/>
@@ -13077,7 +13068,7 @@
     </row>
     <row r="328" spans="1:14">
       <c r="A328" s="22" t="s">
-        <v>403</v>
+        <v>399</v>
       </c>
       <c r="C328" s="22">
         <v>2.8900000000000001E-7</v>
@@ -13090,13 +13081,13 @@
       </c>
       <c r="F328" s="22"/>
       <c r="G328" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H328" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I328" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J328" s="22"/>
       <c r="K328" s="22"/>
@@ -13106,7 +13097,7 @@
     </row>
     <row r="329" spans="1:14">
       <c r="A329" s="22" t="s">
-        <v>404</v>
+        <v>400</v>
       </c>
       <c r="C329" s="22">
         <v>1.9700000000000001E-5</v>
@@ -13119,13 +13110,13 @@
       </c>
       <c r="F329" s="22"/>
       <c r="G329" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H329" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I329" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J329" s="22"/>
       <c r="K329" s="22"/>
@@ -13135,7 +13126,7 @@
     </row>
     <row r="330" spans="1:14">
       <c r="A330" s="22" t="s">
-        <v>405</v>
+        <v>401</v>
       </c>
       <c r="C330" s="22">
         <v>1.19E-6</v>
@@ -13148,13 +13139,13 @@
       </c>
       <c r="F330" s="22"/>
       <c r="G330" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H330" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I330" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J330" s="22"/>
       <c r="K330" s="22"/>
@@ -13164,7 +13155,7 @@
     </row>
     <row r="331" spans="1:14">
       <c r="A331" s="22" t="s">
-        <v>406</v>
+        <v>402</v>
       </c>
       <c r="C331" s="22">
         <v>1.9299999999999999E-7</v>
@@ -13177,13 +13168,13 @@
       </c>
       <c r="F331" s="22"/>
       <c r="G331" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H331" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I331" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J331" s="22"/>
       <c r="K331" s="22"/>
@@ -13193,7 +13184,7 @@
     </row>
     <row r="332" spans="1:14">
       <c r="A332" s="22" t="s">
-        <v>407</v>
+        <v>403</v>
       </c>
       <c r="C332" s="22">
         <v>3.0400000000000001E-6</v>
@@ -13206,13 +13197,13 @@
       </c>
       <c r="F332" s="22"/>
       <c r="G332" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H332" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I332" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J332" s="22"/>
       <c r="K332" s="22"/>
@@ -13222,7 +13213,7 @@
     </row>
     <row r="333" spans="1:14">
       <c r="A333" s="22" t="s">
-        <v>408</v>
+        <v>404</v>
       </c>
       <c r="C333" s="22">
         <v>4.8099999999999997E-6</v>
@@ -13235,13 +13226,13 @@
       </c>
       <c r="F333" s="22"/>
       <c r="G333" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H333" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I333" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J333" s="22"/>
       <c r="K333" s="22"/>
@@ -13251,7 +13242,7 @@
     </row>
     <row r="334" spans="1:14">
       <c r="A334" s="22" t="s">
-        <v>409</v>
+        <v>405</v>
       </c>
       <c r="C334" s="22">
         <v>5.94E-5</v>
@@ -13264,13 +13255,13 @@
       </c>
       <c r="F334" s="22"/>
       <c r="G334" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H334" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I334" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J334" s="22"/>
       <c r="K334" s="22"/>
@@ -13280,7 +13271,7 @@
     </row>
     <row r="335" spans="1:14">
       <c r="A335" s="22" t="s">
-        <v>410</v>
+        <v>406</v>
       </c>
       <c r="C335" s="22">
         <v>3.3700000000000001E-7</v>
@@ -13293,13 +13284,13 @@
       </c>
       <c r="F335" s="22"/>
       <c r="G335" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H335" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I335" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J335" s="22"/>
       <c r="K335" s="22"/>
@@ -13309,7 +13300,7 @@
     </row>
     <row r="336" spans="1:14">
       <c r="A336" s="22" t="s">
-        <v>411</v>
+        <v>407</v>
       </c>
       <c r="C336" s="22">
         <v>1.6800000000000002E-8</v>
@@ -13322,13 +13313,13 @@
       </c>
       <c r="F336" s="22"/>
       <c r="G336" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H336" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I336" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J336" s="22"/>
       <c r="K336" s="22"/>
@@ -13338,7 +13329,7 @@
     </row>
     <row r="337" spans="1:34">
       <c r="A337" s="22" t="s">
-        <v>412</v>
+        <v>408</v>
       </c>
       <c r="C337" s="22">
         <v>5.7800000000000001E-7</v>
@@ -13351,13 +13342,13 @@
       </c>
       <c r="F337" s="22"/>
       <c r="G337" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H337" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I337" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J337" s="22"/>
       <c r="K337" s="22"/>
@@ -13367,7 +13358,7 @@
     </row>
     <row r="338" spans="1:34">
       <c r="A338" s="22" t="s">
-        <v>413</v>
+        <v>409</v>
       </c>
       <c r="C338" s="22">
         <v>2.1699999999999999E-8</v>
@@ -13380,13 +13371,13 @@
       </c>
       <c r="F338" s="22"/>
       <c r="G338" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H338" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I338" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J338" s="22"/>
       <c r="K338" s="22"/>
@@ -13396,7 +13387,7 @@
     </row>
     <row r="339" spans="1:34">
       <c r="A339" s="22" t="s">
-        <v>414</v>
+        <v>410</v>
       </c>
       <c r="C339" s="22">
         <v>3.6099999999999999E-8</v>
@@ -13409,13 +13400,13 @@
       </c>
       <c r="F339" s="22"/>
       <c r="G339" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H339" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I339" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J339" s="22"/>
       <c r="K339" s="22"/>
@@ -13425,7 +13416,7 @@
     </row>
     <row r="340" spans="1:34">
       <c r="A340" s="22" t="s">
-        <v>415</v>
+        <v>411</v>
       </c>
       <c r="C340" s="22">
         <v>2.65E-7</v>
@@ -13438,13 +13429,13 @@
       </c>
       <c r="F340" s="22"/>
       <c r="G340" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H340" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I340" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J340" s="22"/>
       <c r="K340" s="22"/>
@@ -13454,7 +13445,7 @@
     </row>
     <row r="341" spans="1:34">
       <c r="A341" s="22" t="s">
-        <v>416</v>
+        <v>412</v>
       </c>
       <c r="C341" s="22">
         <v>1.1999999999999999E-7</v>
@@ -13467,13 +13458,13 @@
       </c>
       <c r="F341" s="22"/>
       <c r="G341" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H341" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I341" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J341" s="22"/>
       <c r="K341" s="22"/>
@@ -13483,7 +13474,7 @@
     </row>
     <row r="342" spans="1:34">
       <c r="A342" s="22" t="s">
-        <v>417</v>
+        <v>413</v>
       </c>
       <c r="C342" s="22">
         <v>2.6399999999999998E-7</v>
@@ -13496,13 +13487,13 @@
       </c>
       <c r="F342" s="22"/>
       <c r="G342" s="22" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="H342" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I342" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J342" s="22"/>
       <c r="K342" s="22"/>
@@ -13531,7 +13522,7 @@
         <v>15</v>
       </c>
       <c r="I343" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J343" s="22"/>
       <c r="K343" s="22"/>
@@ -13560,7 +13551,7 @@
         <v>15</v>
       </c>
       <c r="I344" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J344" s="22"/>
       <c r="K344" s="22"/>
@@ -13589,7 +13580,7 @@
         <v>15</v>
       </c>
       <c r="I345" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J345" s="22"/>
       <c r="K345" s="22"/>
@@ -13599,7 +13590,7 @@
     </row>
     <row r="346" spans="1:34">
       <c r="A346" s="22" t="s">
-        <v>418</v>
+        <v>414</v>
       </c>
       <c r="C346" s="22">
         <v>9.7499999999999998E-5</v>
@@ -13618,7 +13609,7 @@
         <v>15</v>
       </c>
       <c r="I346" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J346" s="22"/>
       <c r="K346" s="22"/>
@@ -13628,7 +13619,7 @@
     </row>
     <row r="347" spans="1:34">
       <c r="A347" s="22" t="s">
-        <v>419</v>
+        <v>415</v>
       </c>
       <c r="C347" s="22">
         <v>7.5100000000000001E-6</v>
@@ -13647,7 +13638,7 @@
         <v>15</v>
       </c>
       <c r="I347" s="22" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="J347" s="22"/>
       <c r="K347" s="22"/>
@@ -13657,7 +13648,7 @@
     </row>
     <row r="348" spans="1:34">
       <c r="A348" s="22" t="s">
-        <v>420</v>
+        <v>416</v>
       </c>
       <c r="C348" s="22">
         <v>0</v>
@@ -13676,7 +13667,7 @@
         <v>15</v>
       </c>
       <c r="I348" t="s">
-        <v>421</v>
+        <v>417</v>
       </c>
       <c r="J348" s="22"/>
       <c r="K348" s="22"/>
@@ -13740,7 +13731,7 @@
         <v>11</v>
       </c>
       <c r="B351" s="26" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C351" s="25"/>
       <c r="D351" s="26"/>
@@ -13916,10 +13907,10 @@
     </row>
     <row r="361" spans="1:34">
       <c r="A361" s="31" t="s">
-        <v>424</v>
+        <v>420</v>
       </c>
       <c r="B361" s="22" t="s">
-        <v>423</v>
+        <v>419</v>
       </c>
       <c r="C361" s="32">
         <v>1</v>
@@ -14047,7 +14038,7 @@
         <v>11</v>
       </c>
       <c r="B366" s="26" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C366" s="25"/>
       <c r="D366" s="26"/>
@@ -14334,7 +14325,7 @@
         <v>11</v>
       </c>
       <c r="B380" s="26" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C380" s="25"/>
       <c r="D380" s="26"/>
@@ -14594,7 +14585,7 @@
         <v>11</v>
       </c>
       <c r="B392" s="26" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C392" s="25"/>
       <c r="D392" s="26"/>
@@ -15158,7 +15149,7 @@
         <v>11</v>
       </c>
       <c r="B406" s="26" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C406" s="25"/>
       <c r="D406" s="26"/>
@@ -15432,7 +15423,7 @@
         <v>1</v>
       </c>
       <c r="B419" s="24" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C419" s="25"/>
       <c r="D419" s="26"/>
@@ -15472,7 +15463,7 @@
         <v>11</v>
       </c>
       <c r="B420" s="26" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="C420" s="25"/>
       <c r="D420" s="26"/>
@@ -15552,7 +15543,7 @@
         <v>4</v>
       </c>
       <c r="B422" s="26" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C422" s="25"/>
       <c r="D422" s="26"/>
@@ -15672,7 +15663,7 @@
         <v>57</v>
       </c>
       <c r="B425" s="26" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C425" s="25"/>
       <c r="D425" s="29"/>
@@ -15801,10 +15792,10 @@
     </row>
     <row r="428" spans="1:34">
       <c r="A428" s="31" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B428" s="31" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C428" s="32">
         <v>1</v>
@@ -15903,10 +15894,10 @@
     </row>
     <row r="430" spans="1:34">
       <c r="A430" s="31" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B430" s="31" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C430" s="32">
         <v>0</v>
@@ -15953,10 +15944,10 @@
     </row>
     <row r="431" spans="1:34">
       <c r="A431" s="31" t="s">
+        <v>271</v>
+      </c>
+      <c r="B431" s="31" t="s">
         <v>272</v>
-      </c>
-      <c r="B431" s="31" t="s">
-        <v>273</v>
       </c>
       <c r="C431" s="32">
         <v>0</v>
@@ -16003,10 +15994,10 @@
     </row>
     <row r="432" spans="1:34">
       <c r="A432" s="31" t="s">
+        <v>273</v>
+      </c>
+      <c r="B432" s="31" t="s">
         <v>274</v>
-      </c>
-      <c r="B432" s="31" t="s">
-        <v>275</v>
       </c>
       <c r="C432" s="32">
         <v>1</v>
@@ -16053,10 +16044,10 @@
     </row>
     <row r="433" spans="1:34">
       <c r="A433" s="31" t="s">
+        <v>277</v>
+      </c>
+      <c r="B433" s="31" t="s">
         <v>278</v>
-      </c>
-      <c r="B433" s="31" t="s">
-        <v>279</v>
       </c>
       <c r="C433" s="32">
         <v>0</v>
@@ -16103,10 +16094,10 @@
     </row>
     <row r="434" spans="1:34">
       <c r="A434" s="31" t="s">
+        <v>279</v>
+      </c>
+      <c r="B434" s="31" t="s">
         <v>280</v>
-      </c>
-      <c r="B434" s="31" t="s">
-        <v>281</v>
       </c>
       <c r="C434" s="32">
         <v>0</v>
@@ -16153,10 +16144,10 @@
     </row>
     <row r="435" spans="1:34">
       <c r="A435" s="31" t="s">
+        <v>281</v>
+      </c>
+      <c r="B435" s="31" t="s">
         <v>282</v>
-      </c>
-      <c r="B435" s="31" t="s">
-        <v>283</v>
       </c>
       <c r="C435" s="32">
         <v>0</v>
@@ -16175,7 +16166,7 @@
         <v>12</v>
       </c>
       <c r="I435" s="31" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="J435" s="31"/>
       <c r="K435" s="31"/>
@@ -16205,10 +16196,10 @@
     </row>
     <row r="436" spans="1:34">
       <c r="A436" s="31" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="B436" s="31" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="C436" s="32">
         <v>0</v>
@@ -16294,7 +16285,7 @@
         <v>1</v>
       </c>
       <c r="B438" s="24" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C438" s="25"/>
       <c r="D438" s="26"/>
@@ -16334,7 +16325,7 @@
         <v>11</v>
       </c>
       <c r="B439" s="26" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C439" s="25"/>
       <c r="D439" s="26"/>
@@ -16414,7 +16405,7 @@
         <v>4</v>
       </c>
       <c r="B441" s="26" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C441" s="25"/>
       <c r="D441" s="26"/>
@@ -16534,7 +16525,7 @@
         <v>57</v>
       </c>
       <c r="B444" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C444" s="25"/>
       <c r="D444" s="29"/>
@@ -16663,10 +16654,10 @@
     </row>
     <row r="447" spans="1:34">
       <c r="A447" s="31" t="s">
+        <v>273</v>
+      </c>
+      <c r="B447" s="31" t="s">
         <v>274</v>
-      </c>
-      <c r="B447" s="31" t="s">
-        <v>275</v>
       </c>
       <c r="C447" s="32">
         <v>1</v>
@@ -16853,7 +16844,7 @@
         <v>11</v>
       </c>
       <c r="B453" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
     </row>
     <row r="454" spans="1:34">
@@ -16894,7 +16885,7 @@
       </c>
       <c r="B458"/>
     </row>
-    <row r="459" spans="1:34" ht="15.6">
+    <row r="459" spans="1:34" ht="15.75">
       <c r="A459" s="18" t="s">
         <v>7</v>
       </c>
@@ -17067,7 +17058,7 @@
     </row>
     <row r="467" spans="1:9">
       <c r="A467" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B467" s="13" t="s">
         <v>121</v>
@@ -17250,7 +17241,7 @@
         <v>11</v>
       </c>
       <c r="B477" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
     </row>
     <row r="478" spans="1:9">
@@ -17291,7 +17282,7 @@
       </c>
       <c r="B482"/>
     </row>
-    <row r="483" spans="1:9" ht="15.6">
+    <row r="483" spans="1:9" ht="15.75">
       <c r="A483" s="18" t="s">
         <v>7</v>
       </c>
@@ -17464,7 +17455,7 @@
     </row>
     <row r="491" spans="1:9">
       <c r="A491" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B491" s="13" t="s">
         <v>121</v>
@@ -17827,7 +17818,7 @@
         <v>11</v>
       </c>
       <c r="B509" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
     </row>
     <row r="510" spans="1:8">
@@ -17868,7 +17859,7 @@
       </c>
       <c r="B514"/>
     </row>
-    <row r="515" spans="1:9" ht="15.6">
+    <row r="515" spans="1:9" ht="15.75">
       <c r="A515" s="18" t="s">
         <v>7</v>
       </c>
@@ -18041,7 +18032,7 @@
     </row>
     <row r="523" spans="1:9">
       <c r="A523" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B523" s="13" t="s">
         <v>121</v>
@@ -18404,7 +18395,7 @@
         <v>11</v>
       </c>
       <c r="B541" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
     </row>
     <row r="542" spans="1:8">
@@ -18445,7 +18436,7 @@
       </c>
       <c r="B546"/>
     </row>
-    <row r="547" spans="1:9" ht="15.6">
+    <row r="547" spans="1:9" ht="15.75">
       <c r="A547" s="18" t="s">
         <v>7</v>
       </c>
@@ -18618,7 +18609,7 @@
     </row>
     <row r="555" spans="1:9">
       <c r="A555" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B555" s="13" t="s">
         <v>121</v>
@@ -18981,7 +18972,7 @@
         <v>11</v>
       </c>
       <c r="B573" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
     </row>
     <row r="574" spans="1:8">
@@ -19022,7 +19013,7 @@
       </c>
       <c r="B578"/>
     </row>
-    <row r="579" spans="1:9" ht="15.6">
+    <row r="579" spans="1:9" ht="15.75">
       <c r="A579" s="18" t="s">
         <v>7</v>
       </c>
@@ -19195,7 +19186,7 @@
     </row>
     <row r="587" spans="1:9">
       <c r="A587" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B587" s="13" t="s">
         <v>121</v>
@@ -19558,7 +19549,7 @@
         <v>11</v>
       </c>
       <c r="B605" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
     </row>
     <row r="606" spans="1:8">
@@ -19599,7 +19590,7 @@
       </c>
       <c r="B610"/>
     </row>
-    <row r="611" spans="1:9" ht="15.6">
+    <row r="611" spans="1:9" ht="15.75">
       <c r="A611" s="18" t="s">
         <v>7</v>
       </c>
@@ -19772,7 +19763,7 @@
     </row>
     <row r="619" spans="1:9">
       <c r="A619" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B619" s="13" t="s">
         <v>121</v>
@@ -19955,7 +19946,7 @@
         <v>11</v>
       </c>
       <c r="B629" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
     </row>
     <row r="630" spans="1:9">
@@ -19996,7 +19987,7 @@
       </c>
       <c r="B634"/>
     </row>
-    <row r="635" spans="1:9" ht="15.6">
+    <row r="635" spans="1:9" ht="15.75">
       <c r="A635" s="18" t="s">
         <v>7</v>
       </c>
@@ -20169,7 +20160,7 @@
     </row>
     <row r="643" spans="1:9">
       <c r="A643" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B643" s="13" t="s">
         <v>121</v>
@@ -20532,7 +20523,7 @@
         <v>11</v>
       </c>
       <c r="B661" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
     </row>
     <row r="662" spans="1:9">
@@ -20573,7 +20564,7 @@
       </c>
       <c r="B666"/>
     </row>
-    <row r="667" spans="1:9" ht="15.6">
+    <row r="667" spans="1:9" ht="15.75">
       <c r="A667" s="18" t="s">
         <v>7</v>
       </c>
@@ -20746,7 +20737,7 @@
     </row>
     <row r="675" spans="1:9">
       <c r="A675" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B675" s="13" t="s">
         <v>121</v>
@@ -21109,7 +21100,7 @@
         <v>11</v>
       </c>
       <c r="B693" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
     </row>
     <row r="694" spans="1:9">
@@ -21150,7 +21141,7 @@
       </c>
       <c r="B698"/>
     </row>
-    <row r="699" spans="1:9" ht="15.6">
+    <row r="699" spans="1:9" ht="15.75">
       <c r="A699" s="18" t="s">
         <v>7</v>
       </c>
@@ -21323,7 +21314,7 @@
     </row>
     <row r="707" spans="1:9">
       <c r="A707" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B707" s="13" t="s">
         <v>121</v>
@@ -21686,7 +21677,7 @@
         <v>11</v>
       </c>
       <c r="B725" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
     </row>
     <row r="726" spans="1:9">
@@ -21728,7 +21719,7 @@
       </c>
       <c r="B730"/>
     </row>
-    <row r="731" spans="1:9" ht="15.6">
+    <row r="731" spans="1:9" ht="15.75">
       <c r="A731" s="18" t="s">
         <v>7</v>
       </c>
@@ -21901,7 +21892,7 @@
     </row>
     <row r="739" spans="1:9">
       <c r="A739" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B739" s="13" t="s">
         <v>121</v>
@@ -22264,7 +22255,7 @@
         <v>11</v>
       </c>
       <c r="B757" s="13" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
     </row>
     <row r="758" spans="1:21">
@@ -22307,7 +22298,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="763" spans="1:21" ht="15.6">
+    <row r="763" spans="1:21" ht="15.75">
       <c r="A763" s="18" t="s">
         <v>7</v>
       </c>
@@ -22576,10 +22567,10 @@
     </row>
     <row r="770" spans="1:19" s="26" customFormat="1">
       <c r="A770" s="31" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B770" s="31" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C770" s="45">
         <v>1</v>
@@ -23309,7 +23300,7 @@
         <v>11</v>
       </c>
       <c r="B812" s="31" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
     </row>
     <row r="813" spans="1:11" s="26" customFormat="1">
@@ -23417,26 +23408,23 @@
     </row>
     <row r="821" spans="1:9">
       <c r="A821" t="s">
+        <v>479</v>
+      </c>
+      <c r="B821" s="31" t="s">
         <v>259</v>
       </c>
-      <c r="B821" s="31" t="s">
-        <v>260</v>
-      </c>
       <c r="C821" s="46">
-        <v>0.20588960000000001</v>
+        <v>0.1764792</v>
       </c>
       <c r="D821" s="26" t="s">
         <v>35</v>
       </c>
       <c r="E821" s="31"/>
       <c r="G821" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="H821" s="31" t="s">
         <v>12</v>
-      </c>
-      <c r="I821" t="s">
-        <v>304</v>
       </c>
     </row>
     <row r="822" spans="1:9">
@@ -23459,7 +23447,7 @@
         <v>12</v>
       </c>
       <c r="I822" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="823" spans="1:9">
@@ -23468,7 +23456,7 @@
       </c>
       <c r="B823"/>
       <c r="C823" s="21">
-        <v>9.038187058823539E-4</v>
+        <v>6.366155912253407E-4</v>
       </c>
       <c r="D823" t="s">
         <v>13</v>
@@ -23483,7 +23471,7 @@
         <v>15</v>
       </c>
       <c r="I823" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
     </row>
     <row r="824" spans="1:9">
@@ -23492,7 +23480,7 @@
       </c>
       <c r="B824"/>
       <c r="C824" s="21">
-        <v>1.0430494235294118E-2</v>
+        <v>7.346844241170861E-3</v>
       </c>
       <c r="D824" t="s">
         <v>13</v>
@@ -23507,7 +23495,7 @@
         <v>15</v>
       </c>
       <c r="I824" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
     </row>
     <row r="825" spans="1:9" s="49" customFormat="1">
@@ -23518,7 +23506,7 @@
         <v>1</v>
       </c>
       <c r="B826" s="43" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C826" s="25"/>
     </row>
@@ -23527,7 +23515,7 @@
         <v>11</v>
       </c>
       <c r="B827" s="31" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="828" spans="1:9" s="26" customFormat="1">
@@ -23544,7 +23532,7 @@
         <v>4</v>
       </c>
       <c r="B829" s="31" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C829" s="25"/>
     </row>
@@ -23613,10 +23601,10 @@
     </row>
     <row r="835" spans="1:9" s="26" customFormat="1">
       <c r="A835" s="31" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B835" s="31" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C835" s="45">
         <v>1</v>
@@ -23636,27 +23624,23 @@
     </row>
     <row r="836" spans="1:9">
       <c r="A836" t="s">
+        <v>479</v>
+      </c>
+      <c r="B836" s="31" t="s">
         <v>259</v>
       </c>
-      <c r="B836" s="31" t="s">
-        <v>260</v>
-      </c>
       <c r="C836" s="46">
-        <f>0.00593*35.8</f>
-        <v>0.21229399999999998</v>
+        <v>0.1764792</v>
       </c>
       <c r="D836" s="26" t="s">
         <v>35</v>
       </c>
       <c r="E836" s="31"/>
       <c r="G836" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="H836" s="31" t="s">
         <v>12</v>
-      </c>
-      <c r="I836" t="s">
-        <v>307</v>
       </c>
     </row>
     <row r="837" spans="1:9">
@@ -23679,7 +23663,7 @@
         <v>12</v>
       </c>
       <c r="I837" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="838" spans="1:9">
@@ -23688,7 +23672,7 @@
       </c>
       <c r="B838"/>
       <c r="C838" s="13">
-        <v>1.0754999999999999E-2</v>
+        <v>7.5754137849407994E-3</v>
       </c>
       <c r="D838" t="s">
         <v>13</v>
@@ -23703,7 +23687,7 @@
         <v>15</v>
       </c>
       <c r="I838" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
     </row>
     <row r="839" spans="1:9" s="49" customFormat="1">
@@ -23714,7 +23698,7 @@
         <v>1</v>
       </c>
       <c r="B840" s="43" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C840" s="25"/>
       <c r="D840" s="26"/>
@@ -23729,7 +23713,7 @@
         <v>11</v>
       </c>
       <c r="B841" s="31" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C841" s="26"/>
       <c r="D841" s="26"/>
@@ -23856,7 +23840,7 @@
     </row>
     <row r="849" spans="1:9">
       <c r="A849" s="31" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B849" s="31" t="s">
         <v>99</v>
@@ -23878,12 +23862,12 @@
     </row>
     <row r="850" spans="1:9">
       <c r="A850" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B850" s="13" t="s">
-        <v>288</v>
-      </c>
-      <c r="C850">
+        <v>287</v>
+      </c>
+      <c r="C850" s="41">
         <v>0.1764792</v>
       </c>
       <c r="D850" s="26" t="s">
@@ -23896,12 +23880,12 @@
         <v>12</v>
       </c>
       <c r="I850" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="851" spans="1:9">
       <c r="A851" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B851" s="13" t="s">
         <v>99</v>
@@ -23921,7 +23905,7 @@
     </row>
     <row r="852" spans="1:9">
       <c r="A852" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B852" s="13" t="s">
         <v>99</v>
@@ -23941,7 +23925,7 @@
     </row>
     <row r="853" spans="1:9">
       <c r="A853" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B853" s="13" t="s">
         <v>99</v>
@@ -23961,7 +23945,7 @@
     </row>
     <row r="854" spans="1:9">
       <c r="A854" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B854" s="13" t="s">
         <v>99</v>
@@ -23981,7 +23965,7 @@
     </row>
     <row r="855" spans="1:9">
       <c r="A855" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B855" s="13" t="s">
         <v>99</v>
@@ -24001,7 +23985,7 @@
     </row>
     <row r="856" spans="1:9">
       <c r="A856" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B856" s="13" t="s">
         <v>99</v>
@@ -24021,7 +24005,7 @@
     </row>
     <row r="857" spans="1:9">
       <c r="A857" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B857" s="13" t="s">
         <v>99</v>
@@ -24044,7 +24028,7 @@
         <v>84</v>
       </c>
       <c r="C858" s="13">
-        <v>9.6000000000000002E-5</v>
+        <v>6.4625669007360007E-5</v>
       </c>
       <c r="D858" s="26" t="s">
         <v>13</v>
@@ -24060,7 +24044,7 @@
         <v>15</v>
       </c>
       <c r="I858" t="s">
-        <v>308</v>
+        <v>478</v>
       </c>
     </row>
     <row r="859" spans="1:9">
@@ -24068,7 +24052,7 @@
         <v>32</v>
       </c>
       <c r="C859" s="13">
-        <v>3.435E-4</v>
+        <v>2.3123872191696001E-4</v>
       </c>
       <c r="D859" s="26" t="s">
         <v>13</v>
@@ -24084,15 +24068,15 @@
         <v>15</v>
       </c>
       <c r="I859" t="s">
-        <v>308</v>
+        <v>478</v>
       </c>
     </row>
     <row r="860" spans="1:9">
       <c r="A860" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C860" s="13">
-        <v>8.234999999999999E-4</v>
+        <v>5.5436706695375997E-4</v>
       </c>
       <c r="D860" s="26" t="s">
         <v>13</v>
@@ -24108,15 +24092,15 @@
         <v>15</v>
       </c>
       <c r="I860" t="s">
-        <v>308</v>
+        <v>478</v>
       </c>
     </row>
     <row r="861" spans="1:9">
       <c r="A861" t="s">
         <v>86</v>
       </c>
-      <c r="C861" s="13">
-        <v>9.9435000000000009E-3</v>
+      <c r="C861" s="57">
+        <v>6.6938056226529602E-3</v>
       </c>
       <c r="D861" s="26" t="s">
         <v>13</v>
@@ -24131,7 +24115,7 @@
         <v>15</v>
       </c>
       <c r="I861" t="s">
-        <v>308</v>
+        <v>478</v>
       </c>
     </row>
     <row r="862" spans="1:9">
@@ -24139,7 +24123,7 @@
         <v>142</v>
       </c>
       <c r="C862" s="13">
-        <v>7.5000000000000002E-6</v>
+        <v>5.0488803912000003E-6</v>
       </c>
       <c r="D862" s="26" t="s">
         <v>13</v>
@@ -24155,7 +24139,7 @@
         <v>15</v>
       </c>
       <c r="I862" t="s">
-        <v>308</v>
+        <v>478</v>
       </c>
     </row>
     <row r="863" spans="1:9">
@@ -24163,7 +24147,7 @@
         <v>88</v>
       </c>
       <c r="C863" s="13">
-        <v>1.8599999999999999E-4</v>
+        <v>1.2521223370175999E-4</v>
       </c>
       <c r="D863" s="26" t="s">
         <v>13</v>
@@ -24179,7 +24163,7 @@
         <v>15</v>
       </c>
       <c r="I863" t="s">
-        <v>308</v>
+        <v>478</v>
       </c>
     </row>
     <row r="864" spans="1:9">
@@ -24198,7 +24182,7 @@
         <v>1</v>
       </c>
       <c r="B865" s="43" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C865" s="25"/>
       <c r="D865" s="26"/>
@@ -24213,7 +24197,7 @@
         <v>11</v>
       </c>
       <c r="B866" s="31" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C866" s="26"/>
       <c r="D866" s="26"/>
@@ -24288,7 +24272,7 @@
         <v>57</v>
       </c>
       <c r="B871" s="26" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C871" s="25"/>
       <c r="D871" s="29"/>
@@ -24342,7 +24326,7 @@
     </row>
     <row r="874" spans="1:9">
       <c r="A874" s="31" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B874" s="31" t="s">
         <v>170</v>
@@ -24364,7 +24348,7 @@
     </row>
     <row r="875" spans="1:9">
       <c r="A875" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B875" s="31" t="s">
         <v>170</v>
@@ -24398,7 +24382,7 @@
         <v>1</v>
       </c>
       <c r="B877" s="43" t="s">
-        <v>425</v>
+        <v>421</v>
       </c>
       <c r="C877" s="25"/>
       <c r="D877" s="26"/>
@@ -24413,7 +24397,7 @@
         <v>11</v>
       </c>
       <c r="B878" s="31" t="s">
-        <v>426</v>
+        <v>422</v>
       </c>
       <c r="C878" s="26"/>
       <c r="D878" s="26"/>
@@ -24443,7 +24427,7 @@
         <v>4</v>
       </c>
       <c r="B880" s="31" t="s">
-        <v>428</v>
+        <v>424</v>
       </c>
       <c r="C880" s="25"/>
       <c r="D880" s="26"/>
@@ -24473,7 +24457,7 @@
         <v>6</v>
       </c>
       <c r="B882" s="51" t="s">
-        <v>427</v>
+        <v>423</v>
       </c>
       <c r="C882" s="25"/>
       <c r="D882" s="29"/>
@@ -24540,16 +24524,16 @@
     </row>
     <row r="886" spans="1:10">
       <c r="A886" s="43" t="s">
-        <v>425</v>
+        <v>421</v>
       </c>
       <c r="B886" s="31" t="s">
-        <v>428</v>
+        <v>424</v>
       </c>
       <c r="C886" s="26">
         <v>1</v>
       </c>
       <c r="D886" s="26" t="s">
-        <v>427</v>
+        <v>423</v>
       </c>
       <c r="F886" s="24"/>
       <c r="G886" s="31" t="s">
@@ -24571,12 +24555,12 @@
       <c r="H887" s="49"/>
       <c r="I887" s="49"/>
     </row>
-    <row r="888" spans="1:10" ht="15.6">
+    <row r="888" spans="1:10" ht="15.75">
       <c r="A888" s="18" t="s">
         <v>1</v>
       </c>
       <c r="B888" s="43" t="s">
-        <v>430</v>
+        <v>426</v>
       </c>
     </row>
     <row r="889" spans="1:10">
@@ -24603,7 +24587,7 @@
         <v>4</v>
       </c>
       <c r="B891" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
       <c r="F891" s="13"/>
       <c r="J891" s="56"/>
@@ -24633,7 +24617,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="895" spans="1:10" ht="15.6">
+    <row r="895" spans="1:10" ht="15.75">
       <c r="A895" s="18" t="s">
         <v>7</v>
       </c>
@@ -24689,7 +24673,7 @@
         <v>15</v>
       </c>
       <c r="I897" t="s">
-        <v>433</v>
+        <v>429</v>
       </c>
     </row>
     <row r="898" spans="1:9">
@@ -24713,7 +24697,7 @@
         <v>15</v>
       </c>
       <c r="I898" t="s">
-        <v>434</v>
+        <v>430</v>
       </c>
     </row>
     <row r="899" spans="1:9">
@@ -24737,7 +24721,7 @@
         <v>15</v>
       </c>
       <c r="I899" t="s">
-        <v>435</v>
+        <v>431</v>
       </c>
     </row>
     <row r="900" spans="1:9">
@@ -24766,7 +24750,7 @@
     </row>
     <row r="901" spans="1:9">
       <c r="A901" t="s">
-        <v>436</v>
+        <v>432</v>
       </c>
       <c r="B901"/>
       <c r="C901">
@@ -24811,7 +24795,7 @@
     </row>
     <row r="903" spans="1:9">
       <c r="A903" t="s">
-        <v>437</v>
+        <v>433</v>
       </c>
       <c r="B903"/>
       <c r="C903">
@@ -24835,10 +24819,10 @@
     </row>
     <row r="904" spans="1:9">
       <c r="A904" t="s">
-        <v>430</v>
+        <v>426</v>
       </c>
       <c r="B904" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
       <c r="C904">
         <v>1</v>
@@ -24858,7 +24842,7 @@
     </row>
     <row r="905" spans="1:9">
       <c r="A905" t="s">
-        <v>438</v>
+        <v>434</v>
       </c>
       <c r="B905"/>
       <c r="C905">
@@ -24874,12 +24858,12 @@
         <v>12</v>
       </c>
       <c r="I905" t="s">
-        <v>439</v>
+        <v>435</v>
       </c>
     </row>
     <row r="906" spans="1:9">
       <c r="A906" t="s">
-        <v>440</v>
+        <v>436</v>
       </c>
       <c r="B906"/>
       <c r="C906">
@@ -24895,15 +24879,15 @@
         <v>12</v>
       </c>
       <c r="I906" t="s">
-        <v>441</v>
+        <v>437</v>
       </c>
     </row>
     <row r="907" spans="1:9">
       <c r="A907" t="s">
-        <v>442</v>
+        <v>438</v>
       </c>
       <c r="B907" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="C907">
         <v>9.5E-4</v>
@@ -24918,15 +24902,15 @@
         <v>12</v>
       </c>
       <c r="I907" t="s">
-        <v>443</v>
+        <v>439</v>
       </c>
     </row>
     <row r="908" spans="1:9">
       <c r="A908" t="s">
-        <v>445</v>
+        <v>441</v>
       </c>
       <c r="B908" t="s">
-        <v>447</v>
+        <v>443</v>
       </c>
       <c r="C908">
         <v>1.7399999999999999E-5</v>
@@ -24941,15 +24925,15 @@
         <v>12</v>
       </c>
       <c r="I908" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
     </row>
     <row r="909" spans="1:9">
       <c r="A909" t="s">
-        <v>448</v>
+        <v>444</v>
       </c>
       <c r="B909" t="s">
-        <v>450</v>
+        <v>446</v>
       </c>
       <c r="C909">
         <v>5.7600000000000001E-4</v>
@@ -24964,15 +24948,15 @@
         <v>12</v>
       </c>
       <c r="I909" t="s">
-        <v>449</v>
+        <v>445</v>
       </c>
     </row>
     <row r="910" spans="1:9">
       <c r="A910" t="s">
-        <v>478</v>
+        <v>474</v>
       </c>
       <c r="B910" t="s">
-        <v>477</v>
+        <v>473</v>
       </c>
       <c r="C910">
         <v>1.1600000000000001E-11</v>
@@ -24987,7 +24971,7 @@
         <v>12</v>
       </c>
       <c r="I910" t="s">
-        <v>451</v>
+        <v>447</v>
       </c>
     </row>
     <row r="911" spans="1:9">
@@ -25010,7 +24994,7 @@
         <v>12</v>
       </c>
       <c r="I911" t="s">
-        <v>452</v>
+        <v>448</v>
       </c>
     </row>
     <row r="912" spans="1:9">
@@ -25033,7 +25017,7 @@
         <v>12</v>
       </c>
       <c r="I912" t="s">
-        <v>453</v>
+        <v>449</v>
       </c>
     </row>
     <row r="913" spans="1:9">
@@ -25056,15 +25040,15 @@
         <v>12</v>
       </c>
       <c r="I913" t="s">
-        <v>454</v>
+        <v>450</v>
       </c>
     </row>
     <row r="914" spans="1:9">
       <c r="A914" t="s">
-        <v>455</v>
+        <v>451</v>
       </c>
       <c r="B914" t="s">
-        <v>457</v>
+        <v>453</v>
       </c>
       <c r="C914">
         <v>0.1020326</v>
@@ -25079,12 +25063,12 @@
         <v>12</v>
       </c>
       <c r="I914" t="s">
-        <v>456</v>
+        <v>452</v>
       </c>
     </row>
     <row r="915" spans="1:9">
       <c r="A915" t="s">
-        <v>358</v>
+        <v>354</v>
       </c>
       <c r="B915" t="s">
         <v>33</v>
@@ -25096,7 +25080,7 @@
         <v>19</v>
       </c>
       <c r="G915" t="s">
-        <v>458</v>
+        <v>454</v>
       </c>
       <c r="H915" t="s">
         <v>12</v>
@@ -25107,10 +25091,10 @@
     </row>
     <row r="916" spans="1:9">
       <c r="A916" t="s">
-        <v>481</v>
+        <v>477</v>
       </c>
       <c r="B916" t="s">
-        <v>480</v>
+        <v>476</v>
       </c>
       <c r="C916">
         <v>1.1600000000000001E-11</v>
@@ -25119,21 +25103,21 @@
         <v>13</v>
       </c>
       <c r="G916" t="s">
-        <v>459</v>
+        <v>455</v>
       </c>
       <c r="H916" t="s">
         <v>12</v>
       </c>
       <c r="I916" t="s">
-        <v>451</v>
+        <v>447</v>
       </c>
     </row>
     <row r="917" spans="1:9">
       <c r="A917" t="s">
-        <v>460</v>
+        <v>456</v>
       </c>
       <c r="B917" t="s">
-        <v>462</v>
+        <v>458</v>
       </c>
       <c r="C917">
         <v>-2.0200000000000001E-3</v>
@@ -25148,15 +25132,15 @@
         <v>12</v>
       </c>
       <c r="I917" t="s">
-        <v>461</v>
+        <v>457</v>
       </c>
     </row>
     <row r="918" spans="1:9">
       <c r="A918" t="s">
-        <v>463</v>
+        <v>459</v>
       </c>
       <c r="B918" t="s">
-        <v>465</v>
+        <v>461</v>
       </c>
       <c r="C918">
         <v>-1.1600000000000001E-11</v>
@@ -25171,15 +25155,15 @@
         <v>12</v>
       </c>
       <c r="I918" t="s">
-        <v>464</v>
+        <v>460</v>
       </c>
     </row>
     <row r="919" spans="1:9">
       <c r="A919" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
       <c r="B919" t="s">
-        <v>468</v>
+        <v>464</v>
       </c>
       <c r="C919">
         <v>-1.1600000000000001E-11</v>
@@ -25194,15 +25178,15 @@
         <v>12</v>
       </c>
       <c r="I919" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
     </row>
     <row r="920" spans="1:9">
       <c r="A920" t="s">
-        <v>469</v>
+        <v>465</v>
       </c>
       <c r="B920" t="s">
-        <v>471</v>
+        <v>467</v>
       </c>
       <c r="C920">
         <v>-5.63E-5</v>
@@ -25217,15 +25201,15 @@
         <v>12</v>
       </c>
       <c r="I920" t="s">
-        <v>470</v>
+        <v>466</v>
       </c>
     </row>
     <row r="921" spans="1:9">
       <c r="A921" t="s">
-        <v>472</v>
+        <v>468</v>
       </c>
       <c r="B921" t="s">
-        <v>474</v>
+        <v>470</v>
       </c>
       <c r="C921">
         <v>-9.4499999999999998E-4</v>
@@ -25240,15 +25224,15 @@
         <v>12</v>
       </c>
       <c r="I921" t="s">
-        <v>473</v>
+        <v>469</v>
       </c>
     </row>
     <row r="922" spans="1:9">
       <c r="A922" t="s">
-        <v>479</v>
+        <v>475</v>
       </c>
       <c r="B922" t="s">
-        <v>476</v>
+        <v>472</v>
       </c>
       <c r="C922">
         <v>6.28E-6</v>
@@ -25263,15 +25247,15 @@
         <v>12</v>
       </c>
       <c r="I922" t="s">
-        <v>475</v>
+        <v>471</v>
       </c>
     </row>
     <row r="923" spans="1:9">
       <c r="A923" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="B923" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="C923" s="13">
         <v>0.15468000000000001</v>

</xml_diff>

<commit_message>
- Added CO2 to PtG efficiency parameter - Create activity for heat production from biomethane in FR - Updated transport of biomethane by using the newly created activity for heat from biomethane in FR - Updated market for biomethane to account for all biomethane production pathways
</commit_message>
<xml_diff>
--- a/inventories/lci-Tr2050.xlsx
+++ b/inventories/lci-Tr2050.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://engie-my.sharepoint.com/personal/db6421_engie_com/Documents/Documents/GitHub/ADEME_scenarios_premise_gas/inventories/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1759" documentId="13_ncr:1_{6A9A1C53-53B4-4DAF-B82F-70FF83AECA95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D0D3474-BBD2-4870-A7ED-E2183A0A0CA7}"/>
+  <xr:revisionPtr revIDLastSave="1812" documentId="13_ncr:1_{6A9A1C53-53B4-4DAF-B82F-70FF83AECA95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C5960DED-332F-4C3B-BA33-6F8DDDE6C464}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3934" uniqueCount="480">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4115" uniqueCount="484">
   <si>
     <t>Database</t>
   </si>
@@ -1307,9 +1307,6 @@
     <t>Production of refused  derived fuels. It is modelled as a waste to gasification</t>
   </si>
   <si>
-    <t>kg</t>
-  </si>
-  <si>
     <t>RDF, waste</t>
   </si>
   <si>
@@ -1476,6 +1473,21 @@
   </si>
   <si>
     <t>heat production, biomethane, at boiler condensing modulating &lt;100kW</t>
+  </si>
+  <si>
+    <t>Refused derived fuels (not adapted to their LHV)</t>
+  </si>
+  <si>
+    <t>synthetic natural gas from RDF, 70 bar, at plant</t>
+  </si>
+  <si>
+    <t>Synthetic natural gas from RDF, 70 bar, at plant</t>
+  </si>
+  <si>
+    <t>Considered 36% of fossil C-content in refused derived fuels (ADEME Transition 2050 scenarios)</t>
+  </si>
+  <si>
+    <t>refused derived fuels</t>
   </si>
 </sst>
 </file>
@@ -1999,7 +2011,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AH923"/>
+  <dimension ref="A1:AH960"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="73.140625" customWidth="1"/>
@@ -11455,7 +11467,7 @@
         <v>57</v>
       </c>
       <c r="B272" s="31" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="C272" s="22"/>
       <c r="D272" s="22"/>
@@ -23408,7 +23420,7 @@
     </row>
     <row r="821" spans="1:9">
       <c r="A821" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="B821" s="31" t="s">
         <v>259</v>
@@ -23624,7 +23636,7 @@
     </row>
     <row r="836" spans="1:9">
       <c r="A836" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="B836" s="31" t="s">
         <v>259</v>
@@ -24044,7 +24056,7 @@
         <v>15</v>
       </c>
       <c r="I858" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="859" spans="1:9">
@@ -24068,7 +24080,7 @@
         <v>15</v>
       </c>
       <c r="I859" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="860" spans="1:9">
@@ -24092,7 +24104,7 @@
         <v>15</v>
       </c>
       <c r="I860" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="861" spans="1:9">
@@ -24115,7 +24127,7 @@
         <v>15</v>
       </c>
       <c r="I861" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="862" spans="1:9">
@@ -24139,7 +24151,7 @@
         <v>15</v>
       </c>
       <c r="I862" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="863" spans="1:9">
@@ -24163,7 +24175,7 @@
         <v>15</v>
       </c>
       <c r="I863" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="864" spans="1:9">
@@ -24427,7 +24439,7 @@
         <v>4</v>
       </c>
       <c r="B880" s="31" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="C880" s="25"/>
       <c r="D880" s="26"/>
@@ -24456,8 +24468,8 @@
       <c r="A882" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="B882" s="51" t="s">
-        <v>423</v>
+      <c r="B882" t="s">
+        <v>13</v>
       </c>
       <c r="C882" s="25"/>
       <c r="D882" s="29"/>
@@ -24523,17 +24535,17 @@
       </c>
     </row>
     <row r="886" spans="1:10">
-      <c r="A886" s="43" t="s">
+      <c r="A886" s="31" t="s">
         <v>421</v>
       </c>
       <c r="B886" s="31" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="C886" s="26">
         <v>1</v>
       </c>
       <c r="D886" s="26" t="s">
-        <v>423</v>
+        <v>13</v>
       </c>
       <c r="F886" s="24"/>
       <c r="G886" s="31" t="s">
@@ -24560,7 +24572,7 @@
         <v>1</v>
       </c>
       <c r="B888" s="43" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="889" spans="1:10">
@@ -24587,7 +24599,7 @@
         <v>4</v>
       </c>
       <c r="B891" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="F891" s="13"/>
       <c r="J891" s="56"/>
@@ -24673,7 +24685,7 @@
         <v>15</v>
       </c>
       <c r="I897" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="898" spans="1:9">
@@ -24697,7 +24709,7 @@
         <v>15</v>
       </c>
       <c r="I898" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="899" spans="1:9">
@@ -24721,7 +24733,7 @@
         <v>15</v>
       </c>
       <c r="I899" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="900" spans="1:9">
@@ -24750,7 +24762,7 @@
     </row>
     <row r="901" spans="1:9">
       <c r="A901" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="B901"/>
       <c r="C901">
@@ -24795,7 +24807,7 @@
     </row>
     <row r="903" spans="1:9">
       <c r="A903" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="B903"/>
       <c r="C903">
@@ -24819,10 +24831,10 @@
     </row>
     <row r="904" spans="1:9">
       <c r="A904" t="s">
+        <v>425</v>
+      </c>
+      <c r="B904" t="s">
         <v>426</v>
-      </c>
-      <c r="B904" t="s">
-        <v>427</v>
       </c>
       <c r="C904">
         <v>1</v>
@@ -24842,7 +24854,7 @@
     </row>
     <row r="905" spans="1:9">
       <c r="A905" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="B905"/>
       <c r="C905">
@@ -24858,12 +24870,12 @@
         <v>12</v>
       </c>
       <c r="I905" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="906" spans="1:9">
       <c r="A906" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="B906"/>
       <c r="C906">
@@ -24879,15 +24891,15 @@
         <v>12</v>
       </c>
       <c r="I906" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="907" spans="1:9">
       <c r="A907" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="B907" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="C907">
         <v>9.5E-4</v>
@@ -24902,15 +24914,15 @@
         <v>12</v>
       </c>
       <c r="I907" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
     </row>
     <row r="908" spans="1:9">
       <c r="A908" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="B908" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="C908">
         <v>1.7399999999999999E-5</v>
@@ -24925,15 +24937,15 @@
         <v>12</v>
       </c>
       <c r="I908" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
     </row>
     <row r="909" spans="1:9">
       <c r="A909" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B909" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="C909">
         <v>5.7600000000000001E-4</v>
@@ -24948,15 +24960,15 @@
         <v>12</v>
       </c>
       <c r="I909" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
     </row>
     <row r="910" spans="1:9">
       <c r="A910" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="B910" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="C910">
         <v>1.1600000000000001E-11</v>
@@ -24971,7 +24983,7 @@
         <v>12</v>
       </c>
       <c r="I910" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="911" spans="1:9">
@@ -24994,7 +25006,7 @@
         <v>12</v>
       </c>
       <c r="I911" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="912" spans="1:9">
@@ -25017,10 +25029,10 @@
         <v>12</v>
       </c>
       <c r="I912" t="s">
-        <v>449</v>
-      </c>
-    </row>
-    <row r="913" spans="1:9">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="913" spans="1:10">
       <c r="A913" t="s">
         <v>156</v>
       </c>
@@ -25040,15 +25052,15 @@
         <v>12</v>
       </c>
       <c r="I913" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="914" spans="1:10">
+      <c r="A914" t="s">
         <v>450</v>
       </c>
-    </row>
-    <row r="914" spans="1:9">
-      <c r="A914" t="s">
-        <v>451</v>
-      </c>
       <c r="B914" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C914">
         <v>0.1020326</v>
@@ -25063,10 +25075,10 @@
         <v>12</v>
       </c>
       <c r="I914" t="s">
-        <v>452</v>
-      </c>
-    </row>
-    <row r="915" spans="1:9">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="915" spans="1:10">
       <c r="A915" t="s">
         <v>354</v>
       </c>
@@ -25080,7 +25092,7 @@
         <v>19</v>
       </c>
       <c r="G915" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="H915" t="s">
         <v>12</v>
@@ -25089,12 +25101,12 @@
         <v>55</v>
       </c>
     </row>
-    <row r="916" spans="1:9">
+    <row r="916" spans="1:10">
       <c r="A916" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="B916" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="C916">
         <v>1.1600000000000001E-11</v>
@@ -25103,21 +25115,21 @@
         <v>13</v>
       </c>
       <c r="G916" t="s">
+        <v>454</v>
+      </c>
+      <c r="H916" t="s">
+        <v>12</v>
+      </c>
+      <c r="I916" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="917" spans="1:10">
+      <c r="A917" t="s">
         <v>455</v>
       </c>
-      <c r="H916" t="s">
-        <v>12</v>
-      </c>
-      <c r="I916" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="917" spans="1:9">
-      <c r="A917" t="s">
-        <v>456</v>
-      </c>
       <c r="B917" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="C917">
         <v>-2.0200000000000001E-3</v>
@@ -25132,15 +25144,15 @@
         <v>12</v>
       </c>
       <c r="I917" t="s">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="918" spans="1:9">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="918" spans="1:10">
       <c r="A918" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="B918" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="C918">
         <v>-1.1600000000000001E-11</v>
@@ -25155,15 +25167,15 @@
         <v>12</v>
       </c>
       <c r="I918" t="s">
-        <v>460</v>
-      </c>
-    </row>
-    <row r="919" spans="1:9">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="919" spans="1:10">
       <c r="A919" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="B919" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="C919">
         <v>-1.1600000000000001E-11</v>
@@ -25178,15 +25190,15 @@
         <v>12</v>
       </c>
       <c r="I919" t="s">
-        <v>463</v>
-      </c>
-    </row>
-    <row r="920" spans="1:9">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="920" spans="1:10">
       <c r="A920" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="B920" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="C920">
         <v>-5.63E-5</v>
@@ -25201,15 +25213,15 @@
         <v>12</v>
       </c>
       <c r="I920" t="s">
-        <v>466</v>
-      </c>
-    </row>
-    <row r="921" spans="1:9">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="921" spans="1:10">
       <c r="A921" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="B921" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="C921">
         <v>-9.4499999999999998E-4</v>
@@ -25224,15 +25236,15 @@
         <v>12</v>
       </c>
       <c r="I921" t="s">
-        <v>469</v>
-      </c>
-    </row>
-    <row r="922" spans="1:9">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="922" spans="1:10">
       <c r="A922" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="B922" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="C922">
         <v>6.28E-6</v>
@@ -25247,15 +25259,15 @@
         <v>12</v>
       </c>
       <c r="I922" t="s">
-        <v>471</v>
-      </c>
-    </row>
-    <row r="923" spans="1:9">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="923" spans="1:10">
       <c r="A923" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="B923" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="C923" s="13">
         <v>0.15468000000000001</v>
@@ -25268,6 +25280,735 @@
       </c>
       <c r="H923" t="s">
         <v>12</v>
+      </c>
+    </row>
+    <row r="924" spans="1:10">
+      <c r="A924" s="49"/>
+      <c r="B924" s="50"/>
+      <c r="C924" s="49"/>
+      <c r="D924" s="49"/>
+      <c r="E924" s="49"/>
+      <c r="F924" s="49"/>
+      <c r="G924" s="49"/>
+      <c r="H924" s="49"/>
+      <c r="I924" s="49"/>
+    </row>
+    <row r="925" spans="1:10" ht="15.75">
+      <c r="A925" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="B925" s="43" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="926" spans="1:10">
+      <c r="A926" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="B926" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="H926" s="55"/>
+    </row>
+    <row r="927" spans="1:10">
+      <c r="A927" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="B927">
+        <v>1</v>
+      </c>
+      <c r="F927" s="13"/>
+      <c r="H927" s="13"/>
+    </row>
+    <row r="928" spans="1:10">
+      <c r="A928" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="B928" t="s">
+        <v>480</v>
+      </c>
+      <c r="F928" s="13"/>
+      <c r="J928" s="56"/>
+    </row>
+    <row r="929" spans="1:9">
+      <c r="A929" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="B929" t="s">
+        <v>59</v>
+      </c>
+      <c r="F929" s="20"/>
+    </row>
+    <row r="930" spans="1:9">
+      <c r="A930" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="B930" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="931" spans="1:9">
+      <c r="A931" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="B931" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="932" spans="1:9" ht="15.75">
+      <c r="A932" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="B932"/>
+    </row>
+    <row r="933" spans="1:9">
+      <c r="A933" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="B933" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="C933" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="D933" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="E933" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="F933" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="G933" s="30" t="s">
+        <v>2</v>
+      </c>
+      <c r="H933" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="I933" s="27" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="934" spans="1:9">
+      <c r="A934" t="s">
+        <v>138</v>
+      </c>
+      <c r="B934"/>
+      <c r="C934">
+        <f>0.152-C935</f>
+        <v>9.7280000000000005E-2</v>
+      </c>
+      <c r="D934" t="s">
+        <v>13</v>
+      </c>
+      <c r="E934" t="s">
+        <v>83</v>
+      </c>
+      <c r="F934" t="s">
+        <v>25</v>
+      </c>
+      <c r="H934" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="935" spans="1:9">
+      <c r="A935" t="s">
+        <v>32</v>
+      </c>
+      <c r="B935"/>
+      <c r="C935">
+        <f>0.152*0.36</f>
+        <v>5.4719999999999998E-2</v>
+      </c>
+      <c r="D935" t="s">
+        <v>13</v>
+      </c>
+      <c r="E935" t="s">
+        <v>83</v>
+      </c>
+      <c r="F935" t="s">
+        <v>25</v>
+      </c>
+      <c r="H935" t="s">
+        <v>15</v>
+      </c>
+      <c r="I935" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="936" spans="1:9">
+      <c r="A936" t="s">
+        <v>138</v>
+      </c>
+      <c r="B936"/>
+      <c r="C936">
+        <v>1.1100000000000001E-3</v>
+      </c>
+      <c r="D936" t="s">
+        <v>13</v>
+      </c>
+      <c r="E936" t="s">
+        <v>83</v>
+      </c>
+      <c r="F936" t="s">
+        <v>25</v>
+      </c>
+      <c r="H936" t="s">
+        <v>15</v>
+      </c>
+      <c r="I936" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="937" spans="1:9">
+      <c r="A937" t="s">
+        <v>138</v>
+      </c>
+      <c r="B937"/>
+      <c r="C937">
+        <v>1.57E-3</v>
+      </c>
+      <c r="D937" t="s">
+        <v>13</v>
+      </c>
+      <c r="E937" t="s">
+        <v>83</v>
+      </c>
+      <c r="F937" t="s">
+        <v>25</v>
+      </c>
+      <c r="H937" t="s">
+        <v>15</v>
+      </c>
+      <c r="I937" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="938" spans="1:9">
+      <c r="A938" t="s">
+        <v>140</v>
+      </c>
+      <c r="B938"/>
+      <c r="C938">
+        <v>8.1500000000000002E-5</v>
+      </c>
+      <c r="D938" t="s">
+        <v>13</v>
+      </c>
+      <c r="E938" t="s">
+        <v>83</v>
+      </c>
+      <c r="F938" t="s">
+        <v>109</v>
+      </c>
+      <c r="H938" t="s">
+        <v>15</v>
+      </c>
+      <c r="I938" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="939" spans="1:9">
+      <c r="A939" t="s">
+        <v>431</v>
+      </c>
+      <c r="B939"/>
+      <c r="C939">
+        <v>8.9400000000000008E-6</v>
+      </c>
+      <c r="D939" t="s">
+        <v>13</v>
+      </c>
+      <c r="E939" t="s">
+        <v>83</v>
+      </c>
+      <c r="F939" t="s">
+        <v>109</v>
+      </c>
+      <c r="H939" t="s">
+        <v>15</v>
+      </c>
+      <c r="I939" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="940" spans="1:9">
+      <c r="A940" t="s">
+        <v>87</v>
+      </c>
+      <c r="B940"/>
+      <c r="C940">
+        <v>4.6900000000000002E-5</v>
+      </c>
+      <c r="D940" t="s">
+        <v>13</v>
+      </c>
+      <c r="E940" t="s">
+        <v>83</v>
+      </c>
+      <c r="F940" t="s">
+        <v>109</v>
+      </c>
+      <c r="H940" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="941" spans="1:9">
+      <c r="A941" t="s">
+        <v>432</v>
+      </c>
+      <c r="B941"/>
+      <c r="C941">
+        <v>1.2899999999999999E-6</v>
+      </c>
+      <c r="D941" t="s">
+        <v>13</v>
+      </c>
+      <c r="E941" t="s">
+        <v>83</v>
+      </c>
+      <c r="F941" t="s">
+        <v>109</v>
+      </c>
+      <c r="H941" t="s">
+        <v>15</v>
+      </c>
+      <c r="I941" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="942" spans="1:9">
+      <c r="A942" t="s">
+        <v>481</v>
+      </c>
+      <c r="B942" t="s">
+        <v>480</v>
+      </c>
+      <c r="C942">
+        <v>1</v>
+      </c>
+      <c r="D942" t="s">
+        <v>35</v>
+      </c>
+      <c r="G942" t="s">
+        <v>28</v>
+      </c>
+      <c r="H942" t="s">
+        <v>18</v>
+      </c>
+      <c r="I942" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="943" spans="1:9">
+      <c r="A943" t="s">
+        <v>433</v>
+      </c>
+      <c r="B943"/>
+      <c r="C943">
+        <v>1.4500000000000001E-2</v>
+      </c>
+      <c r="D943" t="s">
+        <v>35</v>
+      </c>
+      <c r="G943" t="s">
+        <v>36</v>
+      </c>
+      <c r="H943" t="s">
+        <v>12</v>
+      </c>
+      <c r="I943" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="944" spans="1:9">
+      <c r="A944" t="s">
+        <v>435</v>
+      </c>
+      <c r="B944"/>
+      <c r="C944">
+        <v>4.7200000000000002E-11</v>
+      </c>
+      <c r="D944" t="s">
+        <v>6</v>
+      </c>
+      <c r="G944" t="s">
+        <v>36</v>
+      </c>
+      <c r="H944" t="s">
+        <v>12</v>
+      </c>
+      <c r="I944" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="945" spans="1:9">
+      <c r="A945" t="s">
+        <v>437</v>
+      </c>
+      <c r="B945" t="s">
+        <v>439</v>
+      </c>
+      <c r="C945">
+        <v>9.5E-4</v>
+      </c>
+      <c r="D945" t="s">
+        <v>13</v>
+      </c>
+      <c r="G945" t="s">
+        <v>36</v>
+      </c>
+      <c r="H945" t="s">
+        <v>12</v>
+      </c>
+      <c r="I945" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="946" spans="1:9">
+      <c r="A946" t="s">
+        <v>440</v>
+      </c>
+      <c r="B946" t="s">
+        <v>442</v>
+      </c>
+      <c r="C946">
+        <v>1.7399999999999999E-5</v>
+      </c>
+      <c r="D946" t="s">
+        <v>35</v>
+      </c>
+      <c r="G946" t="s">
+        <v>26</v>
+      </c>
+      <c r="H946" t="s">
+        <v>12</v>
+      </c>
+      <c r="I946" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="947" spans="1:9">
+      <c r="A947" t="s">
+        <v>443</v>
+      </c>
+      <c r="B947" t="s">
+        <v>445</v>
+      </c>
+      <c r="C947">
+        <v>5.7600000000000001E-4</v>
+      </c>
+      <c r="D947" t="s">
+        <v>13</v>
+      </c>
+      <c r="G947" t="s">
+        <v>26</v>
+      </c>
+      <c r="H947" t="s">
+        <v>12</v>
+      </c>
+      <c r="I947" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="948" spans="1:9">
+      <c r="A948" t="s">
+        <v>473</v>
+      </c>
+      <c r="B948" t="s">
+        <v>472</v>
+      </c>
+      <c r="C948">
+        <v>1.1600000000000001E-11</v>
+      </c>
+      <c r="D948" t="s">
+        <v>13</v>
+      </c>
+      <c r="G948" t="s">
+        <v>134</v>
+      </c>
+      <c r="H948" t="s">
+        <v>12</v>
+      </c>
+      <c r="I948" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="949" spans="1:9">
+      <c r="A949" t="s">
+        <v>186</v>
+      </c>
+      <c r="B949" t="s">
+        <v>187</v>
+      </c>
+      <c r="C949">
+        <v>5.3499999999999999E-4</v>
+      </c>
+      <c r="D949" t="s">
+        <v>13</v>
+      </c>
+      <c r="G949" t="s">
+        <v>96</v>
+      </c>
+      <c r="H949" t="s">
+        <v>12</v>
+      </c>
+      <c r="I949" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="950" spans="1:9">
+      <c r="A950" t="s">
+        <v>156</v>
+      </c>
+      <c r="B950" t="s">
+        <v>157</v>
+      </c>
+      <c r="C950">
+        <v>5.6100000000000004E-3</v>
+      </c>
+      <c r="D950" t="s">
+        <v>158</v>
+      </c>
+      <c r="G950" t="s">
+        <v>36</v>
+      </c>
+      <c r="H950" t="s">
+        <v>12</v>
+      </c>
+      <c r="I950" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="951" spans="1:9">
+      <c r="A951" t="s">
+        <v>156</v>
+      </c>
+      <c r="B951" t="s">
+        <v>157</v>
+      </c>
+      <c r="C951">
+        <v>2.7399999999999999E-4</v>
+      </c>
+      <c r="D951" t="s">
+        <v>158</v>
+      </c>
+      <c r="G951" t="s">
+        <v>36</v>
+      </c>
+      <c r="H951" t="s">
+        <v>12</v>
+      </c>
+      <c r="I951" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="952" spans="1:9">
+      <c r="A952" s="31" t="s">
+        <v>483</v>
+      </c>
+      <c r="B952" s="31" t="s">
+        <v>423</v>
+      </c>
+      <c r="C952">
+        <v>0.1020326</v>
+      </c>
+      <c r="D952" t="s">
+        <v>13</v>
+      </c>
+      <c r="G952" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H952" t="s">
+        <v>12</v>
+      </c>
+      <c r="I952" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="953" spans="1:9">
+      <c r="A953" t="s">
+        <v>354</v>
+      </c>
+      <c r="B953" t="s">
+        <v>33</v>
+      </c>
+      <c r="C953">
+        <v>1.77E-2</v>
+      </c>
+      <c r="D953" t="s">
+        <v>19</v>
+      </c>
+      <c r="G953" t="s">
+        <v>453</v>
+      </c>
+      <c r="H953" t="s">
+        <v>12</v>
+      </c>
+      <c r="I953" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="954" spans="1:9">
+      <c r="A954" t="s">
+        <v>476</v>
+      </c>
+      <c r="B954" t="s">
+        <v>475</v>
+      </c>
+      <c r="C954">
+        <v>1.1600000000000001E-11</v>
+      </c>
+      <c r="D954" t="s">
+        <v>13</v>
+      </c>
+      <c r="G954" t="s">
+        <v>454</v>
+      </c>
+      <c r="H954" t="s">
+        <v>12</v>
+      </c>
+      <c r="I954" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="955" spans="1:9">
+      <c r="A955" t="s">
+        <v>455</v>
+      </c>
+      <c r="B955" t="s">
+        <v>457</v>
+      </c>
+      <c r="C955">
+        <v>-2.0200000000000001E-3</v>
+      </c>
+      <c r="D955" t="s">
+        <v>13</v>
+      </c>
+      <c r="G955" t="s">
+        <v>26</v>
+      </c>
+      <c r="H955" t="s">
+        <v>12</v>
+      </c>
+      <c r="I955" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="956" spans="1:9">
+      <c r="A956" t="s">
+        <v>458</v>
+      </c>
+      <c r="B956" t="s">
+        <v>460</v>
+      </c>
+      <c r="C956">
+        <v>-1.1600000000000001E-11</v>
+      </c>
+      <c r="D956" t="s">
+        <v>13</v>
+      </c>
+      <c r="G956" t="s">
+        <v>26</v>
+      </c>
+      <c r="H956" t="s">
+        <v>12</v>
+      </c>
+      <c r="I956" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="957" spans="1:9">
+      <c r="A957" t="s">
+        <v>461</v>
+      </c>
+      <c r="B957" t="s">
+        <v>463</v>
+      </c>
+      <c r="C957">
+        <v>-1.1600000000000001E-11</v>
+      </c>
+      <c r="D957" t="s">
+        <v>13</v>
+      </c>
+      <c r="G957" t="s">
+        <v>26</v>
+      </c>
+      <c r="H957" t="s">
+        <v>12</v>
+      </c>
+      <c r="I957" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="958" spans="1:9">
+      <c r="A958" t="s">
+        <v>464</v>
+      </c>
+      <c r="B958" t="s">
+        <v>466</v>
+      </c>
+      <c r="C958">
+        <v>-5.63E-5</v>
+      </c>
+      <c r="D958" t="s">
+        <v>13</v>
+      </c>
+      <c r="G958" t="s">
+        <v>26</v>
+      </c>
+      <c r="H958" t="s">
+        <v>12</v>
+      </c>
+      <c r="I958" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="959" spans="1:9">
+      <c r="A959" t="s">
+        <v>467</v>
+      </c>
+      <c r="B959" t="s">
+        <v>469</v>
+      </c>
+      <c r="C959">
+        <v>-9.4499999999999998E-4</v>
+      </c>
+      <c r="D959" t="s">
+        <v>13</v>
+      </c>
+      <c r="G959" t="s">
+        <v>26</v>
+      </c>
+      <c r="H959" t="s">
+        <v>12</v>
+      </c>
+      <c r="I959" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="960" spans="1:9">
+      <c r="A960" t="s">
+        <v>474</v>
+      </c>
+      <c r="B960" t="s">
+        <v>471</v>
+      </c>
+      <c r="C960">
+        <v>6.28E-6</v>
+      </c>
+      <c r="D960" t="s">
+        <v>13</v>
+      </c>
+      <c r="G960" t="s">
+        <v>96</v>
+      </c>
+      <c r="H960" t="s">
+        <v>12</v>
+      </c>
+      <c r="I960" t="s">
+        <v>470</v>
       </c>
     </row>
   </sheetData>

</xml_diff>